<commit_message>
chore: reset dashboard and reports to clean production state
</commit_message>
<xml_diff>
--- a/data/reports/viral_posts.xlsx
+++ b/data/reports/viral_posts.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,112 +477,6 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>post_id</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>timestamp</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>image_urls</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>bike storage tent</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>27800</v>
-      </c>
-      <c r="C2" t="n">
-        <v>1700</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2200</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://facebook.com/groups/123/posts/987654321</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Using a bike storage shed as an outdoor kitchen or storage space while camping. Solved all our morning coffee problems!</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Lucas Ethan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>123</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>987654321</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>https://images.unsplash.com/photo-1504280390367-361c6d9f38f4?w=600</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>rv cushion covers</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>350</v>
-      </c>
-      <c r="C3" t="n">
-        <v>42</v>
-      </c>
-      <c r="D3" t="n">
-        <v>18</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://facebook.com/groups/123/posts/123456789</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Way cheaper than replacing the cushions, and when they get dirty, I just throw them in the wash! Best update to our 20-year RV dinette.</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Sarah Connor</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>123</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>123456789</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>https://images.unsplash.com/photo-1523755230320-71a657dcdd76?w=600</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: commercial product scouting, lower reaction threshold to 10+, direct affiliate link extraction, and fix Cloudflare Pages deployment
</commit_message>
<xml_diff>
--- a/data/reports/viral_posts.xlsx
+++ b/data/reports/viral_posts.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P65"/>
+  <dimension ref="A1:Q65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,6 +509,11 @@
           <t>winner_score</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>affiliate_url</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -561,7 +566,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>أجهزة وإلكترونيات (Gadgets &amp; Power)</t>
+          <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -572,6 +577,7 @@
       <c r="P2" t="n">
         <v>99</v>
       </c>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -637,6 +643,7 @@
       <c r="P3" t="n">
         <v>99</v>
       </c>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -698,6 +705,7 @@
       <c r="P4" t="n">
         <v>0</v>
       </c>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -761,6 +769,7 @@
       <c r="P5" t="n">
         <v>91</v>
       </c>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -807,10 +816,23 @@
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/505610137_10228627949544225_29184265896986180_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=p526x296&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=QpbI0HISIwUQ7kNvwGpoC3m&amp;_nc_oc=AdpTak13XLuKr-YWRhmqrvQ1Nfw2nkxBsfWn-qQZc0F0aLf_4Q2FFXtFVQaJYuAkZeU&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQIdd6NLfsBY2RtHLGMrQXjTnSLvFNa0lbB95FHWlJJxeA&amp;oe=6AB39A8F</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>تنظيم وتخزين جاهز (Storage &amp; Organization)</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>bunk bed trampoline ladder</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>97</v>
+      </c>
+      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -875,6 +897,7 @@
       <c r="P7" t="n">
         <v>97</v>
       </c>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -939,6 +962,7 @@
       <c r="P8" t="n">
         <v>89</v>
       </c>
+      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1001,6 +1025,7 @@
       <c r="P9" t="n">
         <v>89</v>
       </c>
+      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1056,7 +1081,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>أجهزة وإلكترونيات (Gadgets &amp; Power)</t>
+          <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1067,6 +1092,7 @@
       <c r="P10" t="n">
         <v>73</v>
       </c>
+      <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1135,6 +1161,7 @@
       <c r="P11" t="n">
         <v>73</v>
       </c>
+      <c r="Q11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1201,6 +1228,7 @@
       <c r="P12" t="n">
         <v>100</v>
       </c>
+      <c r="Q12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1265,6 +1293,7 @@
       <c r="P13" t="n">
         <v>100</v>
       </c>
+      <c r="Q13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1316,7 +1345,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>أجهزة وإلكترونيات (Gadgets &amp; Power)</t>
+          <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1325,8 +1354,9 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>81</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="Q14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1391,6 +1421,7 @@
       <c r="P15" t="n">
         <v>73</v>
       </c>
+      <c r="Q15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1456,6 +1487,7 @@
       <c r="P16" t="n">
         <v>81</v>
       </c>
+      <c r="Q16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1519,6 +1551,7 @@
       <c r="P17" t="n">
         <v>81</v>
       </c>
+      <c r="Q17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1565,10 +1598,19 @@
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/561728600_3814124955386211_4597581507350432745_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=p526x296&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=_H-ynFA0RAEQ7kNvwH652sw&amp;_nc_oc=AdpptTd6DXG4EzDKLZRyUHLG9uCQs_nhT9UV9cTPScoYyv5t3AObH6jdhgh-FP11MNA&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=A1RxZp9G0O8HLhEwpESXLA&amp;_nc_ss=7b2a8&amp;oh=00_AQJSpLc0DrAVWqgXHb9V1F8w2ojb5rgvV8cZ00Tsu2I1oA&amp;oe=6AB3C1B8</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>استبعاد (نقاش/سفر/شكوى)</t>
+        </is>
+      </c>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1629,6 +1671,7 @@
       <c r="P19" t="n">
         <v>0</v>
       </c>
+      <c r="Q19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1693,6 +1736,7 @@
       <c r="P20" t="n">
         <v>83</v>
       </c>
+      <c r="Q20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1755,6 +1799,7 @@
       <c r="P21" t="n">
         <v>91</v>
       </c>
+      <c r="Q21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1807,7 +1852,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>أجهزة وإلكترونيات (Gadgets &amp; Power)</t>
+          <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -1816,8 +1861,9 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>91</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="Q22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1883,6 +1929,7 @@
       <c r="P23" t="n">
         <v>83</v>
       </c>
+      <c r="Q23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1943,6 +1990,7 @@
       <c r="P24" t="n">
         <v>0</v>
       </c>
+      <c r="Q24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2005,6 +2053,7 @@
       <c r="P25" t="n">
         <v>89</v>
       </c>
+      <c r="Q25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2055,10 +2104,23 @@
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/711643338_4031111337187636_2883491981945560264_n.jpg?stp=cp6_dst-jpegr_tt6&amp;cstp=mx2048x1536&amp;ctp=s590x590&amp;_nc_cat=101&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=f_dNgnnJOYgQ7kNvwExjlSF&amp;_nc_oc=AdrWkULW0up9vpUlFyOdOOVFswpvqlDIhNLfoyhWvHBlMRRjGZi30e5xunQe5kh6Z0Q&amp;_nc_zt=23&amp;se=-1&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=ViAqpShX1Nm9L2g-4A-cEw&amp;_nc_ss=7b2a8&amp;oh=00_AQKTSnMNFsMvYlBm6Q9Cs_j26ctmUP0uKKMt38ogPK1CCQ&amp;oe=6AB3BE3A; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/710079281_4031111510520952_7622572342432142030_n.jpg?stp=cp6_dst-jpegr_tt6&amp;cstp=mx1536x2048&amp;ctp=s590x590&amp;_nc_cat=104&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=4dRi6V0TjK4Q7kNvwHSnOiX&amp;_nc_oc=AdrDAS7dm4zU-dcnhVK6W-knhBbh3pssG6jJndvEsBOKEvFfAFNNPsyLOvKMWjs_ivI&amp;_nc_zt=23&amp;se=-1&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=ViAqpShX1Nm9L2g-4A-cEw&amp;_nc_ss=7b2a8&amp;oh=00_AQI6pqkPWZ9WIOjSIkSrF2puVgdYZN4nCE9eR76sArCmFA&amp;oe=6AB3B093</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
+      <c r="M26" t="n">
+        <v>1</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>rv small dehumidifier</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>70</v>
+      </c>
+      <c r="Q26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2127,6 +2189,7 @@
       <c r="P27" t="n">
         <v>70</v>
       </c>
+      <c r="Q27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2194,6 +2257,7 @@
       <c r="P28" t="n">
         <v>81</v>
       </c>
+      <c r="Q28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2259,6 +2323,7 @@
       <c r="P29" t="n">
         <v>81</v>
       </c>
+      <c r="Q29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2306,10 +2371,19 @@
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/778928638_10234377270479258_6720371812830267357_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1206x773&amp;ctp=p180x540&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=2MFpcUQX5nAQ7kNvwGeefCS&amp;_nc_oc=AdpY7NG2vbXAeZdlBhdLZ0XnO1G2KpbNq-q-Vi50uubkYztx7ASFIj4MVK_Shql8qB8&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=A8Me3j8jNja1Mkq3I5rYPg&amp;_nc_ss=7b2a8&amp;oh=00_AQJ-yYB_jczpZmho-tcYD7J0ValNk1dW5sFyRVmDscJnXQ&amp;oe=6AB396CA</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
+      <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>استبعاد (نقاش/سفر/شكوى)</t>
+        </is>
+      </c>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
+      <c r="P30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2371,6 +2445,7 @@
       <c r="P31" t="n">
         <v>0</v>
       </c>
+      <c r="Q31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2435,6 +2510,7 @@
       <c r="P32" t="n">
         <v>81</v>
       </c>
+      <c r="Q32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2497,6 +2573,7 @@
       <c r="P33" t="n">
         <v>81</v>
       </c>
+      <c r="Q33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2557,6 +2634,7 @@
       <c r="P34" t="n">
         <v>0</v>
       </c>
+      <c r="Q34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2619,6 +2697,7 @@
       <c r="P35" t="n">
         <v>81</v>
       </c>
+      <c r="Q35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2669,6 +2748,7 @@
       <c r="P36" t="n">
         <v>0</v>
       </c>
+      <c r="Q36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2721,6 +2801,7 @@
       <c r="P37" t="n">
         <v>0</v>
       </c>
+      <c r="Q37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2773,6 +2854,7 @@
       <c r="P38" t="n">
         <v>0</v>
       </c>
+      <c r="Q38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2815,6 +2897,7 @@
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2865,6 +2948,7 @@
       <c r="P40" t="n">
         <v>0</v>
       </c>
+      <c r="Q40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2917,6 +3001,7 @@
       <c r="P41" t="n">
         <v>0</v>
       </c>
+      <c r="Q41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2969,6 +3054,7 @@
       <c r="P42" t="n">
         <v>0</v>
       </c>
+      <c r="Q42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3011,6 +3097,7 @@
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3069,6 +3156,7 @@
       <c r="P44" t="n">
         <v>0</v>
       </c>
+      <c r="Q44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3129,6 +3217,7 @@
       <c r="P45" t="n">
         <v>0</v>
       </c>
+      <c r="Q45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3182,6 +3271,7 @@
       <c r="P46" t="n">
         <v>0</v>
       </c>
+      <c r="Q46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3233,6 +3323,7 @@
       <c r="P47" t="n">
         <v>0</v>
       </c>
+      <c r="Q47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3244,267 +3335,280 @@
         <v>8</v>
       </c>
       <c r="C48" t="n">
+        <v>48</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/roadtreking/posts/3359003754258580/</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Looking for recommendation on the best route (east to west) through Dallas /Ft Worth.   Midweek, hitting Dallas around Noon.  Pulling 36ft 5th wheel</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>roadtreking</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>3359003754258580</v>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>غير مؤهل (بدون صور)</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>hack</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>8</v>
+      </c>
+      <c r="C49" t="n">
+        <v>32</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/RVhackcamp/posts/4147910648676056/</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Does anyone have a hack for cooling the bottom bunk better? We’ve tried mini fans but they don’t seem to stay upright or stick to the walls very well. I wish we could get an ac vent in there!</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>data\images\hack_4147910648676056\img_1.jpg</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>RVhackcamp</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>4147910648676056</v>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/730771479_10102373262656439_2111230534189182674_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1206x952&amp;ctp=s640x640&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=DGSaV9gAmTAQ7kNvwEywMS_&amp;_nc_oc=AdprvPdL0g_5W2xgZVeuTA___ucidu0kEo0UPwtfNjLrGr8lzJOIt34RmN_8IoOdX94&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=05iOM0uUuQJ8MOIbywV40A&amp;_nc_ss=7b2a8&amp;oh=00_AQJbpgw45n6W01WKIaXHwonMf_0WGJsRiKeyxgsMLPAUaA&amp;oe=6AB3C7D6</t>
+        </is>
+      </c>
+      <c r="M49" t="n">
+        <v>1</v>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>أجهزة وإلكترونيات (Gadgets &amp; Power)</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>rv 12v portable bunk fan</t>
+        </is>
+      </c>
+      <c r="P49" t="n">
+        <v>81</v>
+      </c>
+      <c r="Q49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>amazon find</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>8</v>
+      </c>
+      <c r="C50" t="n">
+        <v>32</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/RVhackcamp/posts/4147910648676056/</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Does anyone have a hack for cooling the bottom bunk better? We’ve tried mini fans but they don’t seem to stay upright or stick to the walls very well. I wish we could get an ac vent in there!</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>data\images\amazon_find_4147910648676056\img_1.jpg</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>RVhackcamp</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>4147910648676056</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/730771479_10102373262656439_2111230534189182674_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1206x952&amp;ctp=s640x640&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=DGSaV9gAmTAQ7kNvwEywMS_&amp;_nc_oc=AdprvPdL0g_5W2xgZVeuTA___ucidu0kEo0UPwtfNjLrGr8lzJOIt34RmN_8IoOdX94&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=-DNXGqSwxAYHz3InfHrB2g&amp;_nc_ss=7b2a8&amp;oh=00_AQKuI7NhSiWUW3pweIYcuSccGm2fBiXhQmnukqpjQKDiRg&amp;oe=6AB3C7D6</t>
+        </is>
+      </c>
+      <c r="M50" t="n">
+        <v>1</v>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>rv 12v portable bunk fan</t>
+        </is>
+      </c>
+      <c r="P50" t="n">
+        <v>81</v>
+      </c>
+      <c r="Q50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>recommendation</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>8</v>
+      </c>
+      <c r="C51" t="n">
+        <v>48</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/roadtreking/posts/3359003754258580/</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Looking for recommendation on the best route (east to west) through Dallas /Ft Worth.   Midweek, hitting Dallas around Noon.  Pulling 36ft 5th wheel</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>roadtreking</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>3359003754258580</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>غير مؤهل (بدون صور)</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>recommendation</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>8</v>
+      </c>
+      <c r="C52" t="n">
         <v>55</v>
       </c>
-      <c r="D48" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" t="inlineStr">
+      <c r="D52" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/roadtreking/posts/3629156827243270/</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>Okay, y’all…we officially did a thing!
 My husband and I just bought our first camper — a 2022 Cherokee Grey Wolf Limited 27RR — and we are COMPLETE newbies to the camping world. We’ve always enjoyed getting away, but this is our first time actually owning a camper, so I’m about to learn A LOT.
 We also have a Can-Am Defender that we can haul in the toy hauler, although we’ll probably use it more for hunting trips than camping.... عرض المزيد</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>roadtreking</t>
-        </is>
-      </c>
-      <c r="J48" t="n">
-        <v>3629156827243270</v>
-      </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="n">
-        <v>0</v>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>غير مؤهل (بدون صور)</t>
-        </is>
-      </c>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>recommendation</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>8</v>
-      </c>
-      <c r="C49" t="n">
-        <v>48</v>
-      </c>
-      <c r="D49" t="n">
-        <v>0</v>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/groups/roadtreking/posts/3359003754258580/</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Looking for recommendation on the best route (east to west) through Dallas /Ft Worth.   Midweek, hitting Dallas around Noon.  Pulling 36ft 5th wheel</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>roadtreking</t>
-        </is>
-      </c>
-      <c r="J49" t="n">
-        <v>3359003754258580</v>
-      </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>amazon find</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>8</v>
-      </c>
-      <c r="C50" t="n">
-        <v>32</v>
-      </c>
-      <c r="D50" t="n">
-        <v>0</v>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/groups/RVhackcamp/posts/4147910648676056/</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Does anyone have a hack for cooling the bottom bunk better? We’ve tried mini fans but they don’t seem to stay upright or stick to the walls very well. I wish we could get an ac vent in there!</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>data\images\amazon_find_4147910648676056\img_1.jpg</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>RVhackcamp</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>4147910648676056</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/730771479_10102373262656439_2111230534189182674_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1206x952&amp;ctp=s640x640&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=DGSaV9gAmTAQ7kNvwEywMS_&amp;_nc_oc=AdprvPdL0g_5W2xgZVeuTA___ucidu0kEo0UPwtfNjLrGr8lzJOIt34RmN_8IoOdX94&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=-DNXGqSwxAYHz3InfHrB2g&amp;_nc_ss=7b2a8&amp;oh=00_AQKuI7NhSiWUW3pweIYcuSccGm2fBiXhQmnukqpjQKDiRg&amp;oe=6AB3C7D6</t>
-        </is>
-      </c>
-      <c r="M50" t="n">
-        <v>1</v>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
-        </is>
-      </c>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>rv 12v portable bunk fan</t>
-        </is>
-      </c>
-      <c r="P50" t="n">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>recommendation</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>8</v>
-      </c>
-      <c r="C51" t="n">
-        <v>48</v>
-      </c>
-      <c r="D51" t="n">
-        <v>0</v>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/groups/roadtreking/posts/3359003754258580/</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Looking for recommendation on the best route (east to west) through Dallas /Ft Worth.   Midweek, hitting Dallas around Noon.  Pulling 36ft 5th wheel</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>roadtreking</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>3359003754258580</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="n">
-        <v>0</v>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>غير مؤهل (بدون صور)</t>
-        </is>
-      </c>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>hack</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>8</v>
-      </c>
-      <c r="C52" t="n">
-        <v>32</v>
-      </c>
-      <c r="D52" t="n">
-        <v>0</v>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/groups/RVhackcamp/posts/4147910648676056/</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>Does anyone have a hack for cooling the bottom bunk better? We’ve tried mini fans but they don’t seem to stay upright or stick to the walls very well. I wish we could get an ac vent in there!</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>data\images\hack_4147910648676056\img_1.jpg</t>
-        </is>
-      </c>
+      <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>RVhackcamp</t>
+          <t>roadtreking</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>4147910648676056</v>
+        <v>3629156827243270</v>
       </c>
       <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/730771479_10102373262656439_2111230534189182674_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1206x952&amp;ctp=s640x640&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=DGSaV9gAmTAQ7kNvwEywMS_&amp;_nc_oc=AdprvPdL0g_5W2xgZVeuTA___ucidu0kEo0UPwtfNjLrGr8lzJOIt34RmN_8IoOdX94&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=05iOM0uUuQJ8MOIbywV40A&amp;_nc_ss=7b2a8&amp;oh=00_AQJbpgw45n6W01WKIaXHwonMf_0WGJsRiKeyxgsMLPAUaA&amp;oe=6AB3C7D6</t>
-        </is>
-      </c>
+      <c r="L52" t="inlineStr"/>
       <c r="M52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>أجهزة وإلكترونيات (Gadgets &amp; Power)</t>
-        </is>
-      </c>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t>rv 12v portable bunk fan</t>
-        </is>
-      </c>
+          <t>غير مؤهل (بدون صور)</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr"/>
       <c r="P52" t="n">
-        <v>81</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3559,6 +3663,7 @@
       <c r="P53" t="n">
         <v>0</v>
       </c>
+      <c r="Q53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3570,30 +3675,30 @@
         <v>7</v>
       </c>
       <c r="C54" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/roadtreking/posts/3617867058372247/</t>
+          <t>https://www.facebook.com/groups/RVhackcamp/posts/3128604820606649/</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Hello, has anyone ever paid to have someone move their RV from one state to another? I was looking online but now I have been bombarded by different companies. Just hoping to hear if someone has used one. ￼</t>
+          <t>Looking for campground recommendations for Corpus Christi, TX.</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
-          <t>roadtreking</t>
+          <t>RVhackcamp</t>
         </is>
       </c>
       <c r="J54" t="n">
-        <v>3617867058372247</v>
+        <v>3128604820606649</v>
       </c>
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
@@ -3609,6 +3714,7 @@
       <c r="P54" t="n">
         <v>0</v>
       </c>
+      <c r="Q54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3620,37 +3726,46 @@
         <v>7</v>
       </c>
       <c r="C55" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D55" t="n">
         <v>0</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/RVhackcamp/posts/3128604820606649/</t>
+          <t>https://www.facebook.com/groups/roadtreking/posts/3617867058372247/</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Looking for campground recommendations for Corpus Christi, TX.</t>
+          <t>Hello, has anyone ever paid to have someone move their RV from one state to another? I was looking online but now I have been bombarded by different companies. Just hoping to hear if someone has used one. ￼</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
-          <t>RVhackcamp</t>
+          <t>roadtreking</t>
         </is>
       </c>
       <c r="J55" t="n">
-        <v>3128604820606649</v>
+        <v>3617867058372247</v>
       </c>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
+      <c r="M55" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>غير مؤهل (بدون صور)</t>
+        </is>
+      </c>
       <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
+      <c r="P55" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3703,6 +3818,7 @@
       <c r="P56" t="n">
         <v>0</v>
       </c>
+      <c r="Q56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3755,6 +3871,7 @@
       <c r="P57" t="n">
         <v>0</v>
       </c>
+      <c r="Q57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3807,6 +3924,7 @@
       <c r="P58" t="n">
         <v>0</v>
       </c>
+      <c r="Q58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3857,6 +3975,7 @@
       <c r="P59" t="n">
         <v>0</v>
       </c>
+      <c r="Q59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3905,21 +4024,18 @@
         </is>
       </c>
       <c r="M60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>إكسسوارات وحلول ذكية (Smart Accessories &amp; Hacks)</t>
-        </is>
-      </c>
-      <c r="O60" t="inlineStr">
-        <is>
-          <t>rv collapsible pet pool</t>
-        </is>
-      </c>
+          <t>استبعاد (نقاش/سفر/شكوى)</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr"/>
       <c r="P60" t="n">
-        <v>100</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3981,6 +4097,7 @@
       <c r="P61" t="n">
         <v>0</v>
       </c>
+      <c r="Q61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4041,6 +4158,7 @@
       <c r="P62" t="n">
         <v>0</v>
       </c>
+      <c r="Q62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4091,6 +4209,7 @@
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4142,7 +4261,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>أجهزة وإلكترونيات (Gadgets &amp; Power)</t>
+          <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
@@ -4151,8 +4270,9 @@
         </is>
       </c>
       <c r="P64" t="n">
-        <v>86</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="Q64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4217,6 +4337,7 @@
       <c r="P65" t="n">
         <v>70</v>
       </c>
+      <c r="Q65" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: deep group feed crawling (40 scrolls/100 posts limit), physical wheel scrolling, and post copywriter
</commit_message>
<xml_diff>
--- a/data/reports/viral_posts.xlsx
+++ b/data/reports/viral_posts.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q65"/>
+  <dimension ref="A1:R65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,55 +461,60 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>generated_caption</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>local_images</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>author</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>group_id</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>post_id</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>timestamp</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>image_urls</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>is_product</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>product_category</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>amazon_query</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>winner_score</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>affiliate_url</t>
         </is>
@@ -543,41 +548,47 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>Honestly didn't expect rv must have gadget to work this well, but it literally solved the problem on our last trip! Best purchase I've made in a while.
+I left the direct link in the first comment for anyone who needs it 👇</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>data\images\must_have_gadget_4124414001025721\img_1.jpg; data\images\must_have_gadget_4124414001025721\img_2.jpg; data\images\must_have_gadget_4124414001025721\img_3.jpg</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>4124414001025721</v>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/714611806_10215958763359663_6601841730117456563_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1386x2048&amp;ctp=s590x590&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=e1O3zMI2FBAQ7kNvwH0f9kz&amp;_nc_oc=Adrlw0O8ab8aboNq_-Issv4ZciryIkKZBDfmyzFxZiGWadT3Gk3TKsaWld3S8OPoobk&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=xdIPSj7R-3lhEMKdb3QlGQ&amp;_nc_ss=7b2a8&amp;oh=00_AQI4ZelcCflvqEJ2kpSSxWFEzejtqTMDMQQyV93rqWUKtQ&amp;oe=6AB3BC85; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/714384150_10215958763759673_8245354785028741008_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx935x1272&amp;ctp=s590x590&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=FpOY9vQtJ6YQ7kNvwGRrp_C&amp;_nc_oc=AdqVcmZxnd_HmBnrMWMo1IQwxCZhT3KzI9F-kZeoGmuIlDtWr_BOud5c2P1J1ogRNTQ&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=xdIPSj7R-3lhEMKdb3QlGQ&amp;_nc_ss=7b2a8&amp;oh=00_AQLJppTjdJa-7osH0NPYnAJCp__ERaaJzgRYx4xQGpdzUA&amp;oe=6AB39A9B; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/715435401_10215958764119682_4239662220553189837_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx2048x2048&amp;ctp=s590x590&amp;_nc_cat=101&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=Lgyxk1qwPP8Q7kNvwExOJLi&amp;_nc_oc=AdrFTRRleOoNTZXioS5hSn97k-U5pLE8wzdP2Th_-pYVRRRQHaSxcAxUNJWUmBCyl3Y&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=xdIPSj7R-3lhEMKdb3QlGQ&amp;_nc_ss=7b2a8&amp;oh=00_AQKXWP-_umRYvMmKVNdu03tTuOXsQLCnkNnzHA-iQQCm2w&amp;oe=6AB3B4D0</t>
         </is>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>1</v>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>rv must have gadget</t>
         </is>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>99</v>
       </c>
-      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -607,43 +618,50 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>Our teenager flat-out refused to squeeze into the standard RV bunk until we set this up.
+It turned a tiny, cramped corner into her own cozy private space in less than five minutes. Honestly saved our whole family camping trip!
+I dropped the link in the first comment if you want one 👇</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>data\images\must_have_gadget_4124414001025721\img_1.jpg; data\images\must_have_gadget_4124414001025721\img_2.jpg; data\images\must_have_gadget_4124414001025721\img_3.jpg</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>4124414001025721</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/714611806_10215958763359663_6601841730117456563_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1386x2048&amp;ctp=s590x590&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=e1O3zMI2FBAQ7kNvwH0f9kz&amp;_nc_oc=Adrlw0O8ab8aboNq_-Issv4ZciryIkKZBDfmyzFxZiGWadT3Gk3TKsaWld3S8OPoobk&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=xdIPSj7R-3lhEMKdb3QlGQ&amp;_nc_ss=7b2a8&amp;oh=00_AQI4ZelcCflvqEJ2kpSSxWFEzejtqTMDMQQyV93rqWUKtQ&amp;oe=6AB3BC85; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/714384150_10215958763759673_8245354785028741008_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx935x1272&amp;ctp=s590x590&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=FpOY9vQtJ6YQ7kNvwGRrp_C&amp;_nc_oc=AdqVcmZxnd_HmBnrMWMo1IQwxCZhT3KzI9F-kZeoGmuIlDtWr_BOud5c2P1J1ogRNTQ&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=xdIPSj7R-3lhEMKdb3QlGQ&amp;_nc_ss=7b2a8&amp;oh=00_AQLJppTjdJa-7osH0NPYnAJCp__ERaaJzgRYx4xQGpdzUA&amp;oe=6AB39A9B; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/715435401_10215958764119682_4239662220553189837_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx2048x2048&amp;ctp=s590x590&amp;_nc_cat=101&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=Lgyxk1qwPP8Q7kNvwExOJLi&amp;_nc_oc=AdrFTRRleOoNTZXioS5hSn97k-U5pLE8wzdP2Th_-pYVRRRQHaSxcAxUNJWUmBCyl3Y&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=xdIPSj7R-3lhEMKdb3QlGQ&amp;_nc_ss=7b2a8&amp;oh=00_AQKXWP-_umRYvMmKVNdu03tTuOXsQLCnkNnzHA-iQQCm2w&amp;oe=6AB3B4D0</t>
         </is>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>1</v>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>rv must have gadget</t>
         </is>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>99</v>
       </c>
-      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -671,41 +689,42 @@
 We are so happy!!</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
         <is>
           <t>data\images\hack_2389439124523226\img_1.jpg; data\images\hack_2389439124523226\img_2.jpg; data\images\hack_2389439124523226\img_3.jpg; data\images\hack_2389439124523226\img_4.jpg; data\images\hack_2389439124523226\img_5.jpg</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2389439124523226</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t1.6435-9/189573366_4439537905141_7744078254309363716_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx960x960&amp;ctp=s590x590&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=33274f&amp;_nc_ohc=aBBTZz_R2QQQ7kNvwH6lixB&amp;_nc_oc=AdrDHARpuJPd1FYGMfbWaoFRCYKM68UoRfG2ibtABAbasTot0CRQZOaJ-tsq3z4hwBg&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQJPkyXCbdYJpNgWBF9bziSrMSwlVo0YIakXWfqgEwrXJw&amp;oe=6AD55F0B; https://scontent.fcai19-4.fna.fbcdn.net/v/t1.6435-9/189465542_4439538025144_4331371041119588443_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx960x960&amp;ctp=s590x590&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=33274f&amp;_nc_ohc=KbayQGqGrwcQ7kNvwFlrRoi&amp;_nc_oc=AdpEpEsUlvAoi8JLc4pIs1f5SOVBqvi4Pm3eVx7zeZzXdA8uqeXg2rlvBqel-3gkqVU&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQIuIceKOeu1P6QBrOiEmSKpFEGQBXZvQCoMTZQw_bvZeA&amp;oe=6AD542BC; https://scontent.fcai19-4.fna.fbcdn.net/v/t1.6435-9/187248079_4439538905166_2897692911484219363_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx960x960&amp;ctp=s590x590&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=33274f&amp;_nc_ohc=Hsd1zRsnrtUQ7kNvwHCNVF0&amp;_nc_oc=AdpkHDrkX41B23eqN97JnQ7_e-0FiKex0OUAcnQ4kC7GgOAyRVIqGhm2dJ13fdumL6s&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQJhNpn4ODMfW5R59eS_i0Qj61CzeETc7Jl8XQMBU08bRA&amp;oe=6AD54DE9; https://scontent.fcai19-4.fna.fbcdn.net/v/t1.6435-9/189239174_4439538665160_1105640096963475063_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx960x960&amp;ctp=s590x590&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=33274f&amp;_nc_ohc=aQ_AFWigRS0Q7kNvwEm6Wlv&amp;_nc_oc=AdoELA5q9-3ZXPZ-v-HOrHuCoCzgBgw9dTspmR43JLg06-Jjd_0mw6pYPx3F7dipSXw&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQLUjhCUBhH1_IlA3T75xQf_syW9hZRdYJWgHGXkW-YOxw&amp;oe=6AD55CF8; https://scontent.fcai19-4.fna.fbcdn.net/v/t1.6435-9/189573366_4439538465155_4433609016928526357_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx960x960&amp;ctp=s590x590&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=33274f&amp;_nc_ohc=q7E8f_9ooVYQ7kNvwFH7NPn&amp;_nc_oc=AdoqHlvmXZ36vOEywV086n7ThG1SXJfZXcCcsBrMGB03C0jais65-Ei56dleFzvx710&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQIwEVuMu05e-pZfNXH7FQtqaJfq2B-xgk1w4vnodfMNkQ&amp;oe=6AD5530E</t>
         </is>
       </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" t="inlineStr">
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr">
         <is>
           <t>استبعاد (نقاش/سفر/شكوى)</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -733,43 +752,44 @@
 We are so happy!!</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
         <is>
           <t>data\images\hack_2389439124523226\img_1.jpg; data\images\hack_2389439124523226\img_2.jpg; data\images\hack_2389439124523226\img_3.jpg; data\images\hack_2389439124523226\img_4.jpg; data\images\hack_2389439124523226\img_5.jpg</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>2389439124523226</v>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t1.6435-9/189573366_4439537905141_7744078254309363716_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx960x960&amp;ctp=s590x590&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=33274f&amp;_nc_ohc=aBBTZz_R2QQQ7kNvwH6lixB&amp;_nc_oc=AdrDHARpuJPd1FYGMfbWaoFRCYKM68UoRfG2ibtABAbasTot0CRQZOaJ-tsq3z4hwBg&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQJPkyXCbdYJpNgWBF9bziSrMSwlVo0YIakXWfqgEwrXJw&amp;oe=6AD55F0B; https://scontent.fcai19-4.fna.fbcdn.net/v/t1.6435-9/189465542_4439538025144_4331371041119588443_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx960x960&amp;ctp=s590x590&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=33274f&amp;_nc_ohc=KbayQGqGrwcQ7kNvwFlrRoi&amp;_nc_oc=AdpEpEsUlvAoi8JLc4pIs1f5SOVBqvi4Pm3eVx7zeZzXdA8uqeXg2rlvBqel-3gkqVU&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQIuIceKOeu1P6QBrOiEmSKpFEGQBXZvQCoMTZQw_bvZeA&amp;oe=6AD542BC; https://scontent.fcai19-4.fna.fbcdn.net/v/t1.6435-9/187248079_4439538905166_2897692911484219363_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx960x960&amp;ctp=s590x590&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=33274f&amp;_nc_ohc=Hsd1zRsnrtUQ7kNvwHCNVF0&amp;_nc_oc=AdpkHDrkX41B23eqN97JnQ7_e-0FiKex0OUAcnQ4kC7GgOAyRVIqGhm2dJ13fdumL6s&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQJhNpn4ODMfW5R59eS_i0Qj61CzeETc7Jl8XQMBU08bRA&amp;oe=6AD54DE9; https://scontent.fcai19-4.fna.fbcdn.net/v/t1.6435-9/189239174_4439538665160_1105640096963475063_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx960x960&amp;ctp=s590x590&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=33274f&amp;_nc_ohc=aQ_AFWigRS0Q7kNvwEm6Wlv&amp;_nc_oc=AdoELA5q9-3ZXPZ-v-HOrHuCoCzgBgw9dTspmR43JLg06-Jjd_0mw6pYPx3F7dipSXw&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQLUjhCUBhH1_IlA3T75xQf_syW9hZRdYJWgHGXkW-YOxw&amp;oe=6AD55CF8; https://scontent.fcai19-4.fna.fbcdn.net/v/t1.6435-9/189573366_4439538465155_4433609016928526357_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx960x960&amp;ctp=s590x590&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=33274f&amp;_nc_ohc=q7E8f_9ooVYQ7kNvwFH7NPn&amp;_nc_oc=AdoqHlvmXZ36vOEywV086n7ThG1SXJfZXcCcsBrMGB03C0jais65-Ei56dleFzvx710&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQIwEVuMu05e-pZfNXH7FQtqaJfq2B-xgk1w4vnodfMNkQ&amp;oe=6AD5530E</t>
         </is>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>1</v>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>إكسسوارات وحلول ذكية (Smart Accessories &amp; Hacks)</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>rv hack</t>
         </is>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>91</v>
       </c>
-      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -798,41 +818,47 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>Honestly didn't expect bunk bed trampoline ladder to work this well, but it literally solved the problem on our last trip! Best purchase I've made in a while.
+I left the direct link in the first comment for anyone who needs it 👇</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>data\images\hack_3308082032658926\img_1.jpg</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>3308082032658926</v>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/505610137_10228627949544225_29184265896986180_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=p526x296&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=QpbI0HISIwUQ7kNvwGpoC3m&amp;_nc_oc=AdpTak13XLuKr-YWRhmqrvQ1Nfw2nkxBsfWn-qQZc0F0aLf_4Q2FFXtFVQaJYuAkZeU&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQIdd6NLfsBY2RtHLGMrQXjTnSLvFNa0lbB95FHWlJJxeA&amp;oe=6AB39A8F</t>
         </is>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>1</v>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>تنظيم وتخزين جاهز (Storage &amp; Organization)</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>bunk bed trampoline ladder</t>
         </is>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>97</v>
       </c>
-      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -861,43 +887,50 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>Best $25 camper hack we’ve done so far.
+Our camper didn’t come with a bunk ladder, and my girls kept struggling to climb up. Regular ones were way too tall, but a cheap trampoline ladder hooked right onto the frame.
+I’ll leave the link in the first comment! 👇</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>data\images\hack_3308082032658926\img_1.jpg</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>3308082032658926</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/505610137_10228627949544225_29184265896986180_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=p526x296&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=QpbI0HISIwUQ7kNvwGpoC3m&amp;_nc_oc=AdpTak13XLuKr-YWRhmqrvQ1Nfw2nkxBsfWn-qQZc0F0aLf_4Q2FFXtFVQaJYuAkZeU&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQIdd6NLfsBY2RtHLGMrQXjTnSLvFNa0lbB95FHWlJJxeA&amp;oe=6AB39A8F</t>
         </is>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>1</v>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>تنظيم وتخزين جاهز (Storage &amp; Organization)</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>bunk bed trampoline ladder</t>
         </is>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>97</v>
       </c>
-      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -926,43 +959,50 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>Honestly, why did no one tell me about this before our last RV trip?
+I used to spend 20 minutes stressing over getting the rig level on uneven ground every time we parked. Got this last week and was fully set up in under two minutes flat.
+I left the link in the first comment if you want it! 👇</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>data\images\must_have_gadget_4009327692534353\img_1.jpg</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>4009327692534353</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/643396407_10238655093303438_2982570874296650007_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx2048x1536&amp;ctp=s720x720&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=QvAD0_ZeHdEQ7kNvwHy778z&amp;_nc_oc=AdqBe3rZBJ3X2Tj7tMqgAfl7NMUdiQQd8sMoyfXjYeHH-8ewyBv_yNBoyhPsZucF3yA&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=1eCUd6gOywCURufMd_fVdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQIUChpHh0PDussfNot-ZthDMoiDU_kAzhX2nuuDxqd_Xg&amp;oe=6AB3C10F</t>
         </is>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>1</v>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>rv must have gadget</t>
         </is>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>89</v>
       </c>
-      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -989,43 +1029,44 @@
           <t>What’s your “why did no one tell me I needed this?” item for camping?... عرض المزيد</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
         <is>
           <t>data\images\must_have_gadget_4009327692534353\img_1.jpg</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
         <v>4009327692534353</v>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr">
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/643396407_10238655093303438_2982570874296650007_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx2048x1536&amp;ctp=s720x720&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=QvAD0_ZeHdEQ7kNvwHy778z&amp;_nc_oc=AdqBe3rZBJ3X2Tj7tMqgAfl7NMUdiQQd8sMoyfXjYeHH-8ewyBv_yNBoyhPsZucF3yA&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=1eCUd6gOywCURufMd_fVdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQIUChpHh0PDussfNot-ZthDMoiDU_kAzhX2nuuDxqd_Xg&amp;oe=6AB3C10F</t>
         </is>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>1</v>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات (Gadgets &amp; Power)</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>rv must have gadget</t>
         </is>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
         <v>89</v>
       </c>
-      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1058,41 +1099,47 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>Honestly didn't expect rv amazon find to work this well, but it literally solved the problem on our last trip! Best purchase I've made in a while.
+I left the direct link in the first comment for anyone who needs it 👇</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>data\images\amazon_find_4113730608760727\img_1.jpg</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
         <v>4113730608760727</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr">
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/710710608_3365719276935810_913380809031877934_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1290x1728&amp;ctp=p526x296&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=W4Mx_7udmmcQ7kNvwFJ4xZI&amp;_nc_oc=AdqFT1td-gxh5OjykSM57gmwHH8rg2J4DkAgoVkCftj1D8ioDF6ymqGPV7zwA4SlLIs&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=-DNXGqSwxAYHz3InfHrB2g&amp;_nc_ss=7b2a8&amp;oh=00_AQJVruWyQvhPwbT7S7oAFjSG9T7OumAe5miDQecXxPLwqw&amp;oe=6AB3B1EB</t>
         </is>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>1</v>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>rv amazon find</t>
         </is>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>73</v>
       </c>
-      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1125,43 +1172,50 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>Finally figured out how to block that blinding morning sun in our RV.
+I grabbed this cheap blackout vinyl on Amazon, and it completely hides the ugly window frames while keeping the camper pitch black for sleeping in. 
+I left the link in the first comment 👇</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>data\images\amazon_find_4113730608760727\img_1.jpg</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>4113730608760727</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr">
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/710710608_3365719276935810_913380809031877934_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1290x1728&amp;ctp=p526x296&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=W4Mx_7udmmcQ7kNvwFJ4xZI&amp;_nc_oc=AdqFT1td-gxh5OjykSM57gmwHH8rg2J4DkAgoVkCftj1D8ioDF6ymqGPV7zwA4SlLIs&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=-DNXGqSwxAYHz3InfHrB2g&amp;_nc_ss=7b2a8&amp;oh=00_AQJVruWyQvhPwbT7S7oAFjSG9T7OumAe5miDQecXxPLwqw&amp;oe=6AB3B1EB</t>
         </is>
       </c>
-      <c r="M11" t="n">
+      <c r="N11" t="n">
         <v>1</v>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>rv amazon find</t>
         </is>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>73</v>
       </c>
-      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1192,43 +1246,49 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>Honestly didn't expect rv hanging shoe organizer to work this well, but it literally solved the problem on our last trip! Best purchase I've made in a while.
+I left the direct link in the first comment for anyone who needs it 👇</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>data\images\must_have_gadget_177043908\img_1.jpg; data\images\must_have_gadget_177043908\img_2.jpg; data\images\must_have_gadget_177043908\img_3.jpg; data\images\must_have_gadget_177043908\img_4.jpg; data\images\must_have_gadget_177043908\img_5.jpg</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
         <is>
           <t>Public Search</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>177043908</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr">
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/655900116_26426801810294266_616338587343076791_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx736x1000&amp;ctp=s590x590&amp;_nc_cat=103&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=jB-xL4WCwAgQ7kNvwFsIIDC&amp;_nc_oc=AdoGV6P4nAjOyR8A4bqzpg8FsSFsTzuA9J9oYzN3nvHnZSZOlC6sXJaEQPLvrs9zuXc&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=UnTMyOwTXyTerwvTKQdb8A&amp;_nc_ss=7b2a8&amp;oh=00_AQLUYw_U16e1OluoKTx7qceTxgRUASaIWKPWYSNAPF7z1w&amp;oe=6AB3AB8A; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/656840747_26426801883627592_1775700405554872607_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx736x1000&amp;ctp=s590x590&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=j8NFBjoOyBgQ7kNvwGMUo7s&amp;_nc_oc=AdqOeMpnaO7GTgDmhNWFl03ZZ_QL7ZHss7jWCq2a7ZYSMXuKGE1WUJ9CfjqRoFvo9eU&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=UnTMyOwTXyTerwvTKQdb8A&amp;_nc_ss=7b2a8&amp;oh=00_AQJRDiTDfLxEoM8Xrvq6SX0XMQ3iNan62a_aWFxF6SNbTQ&amp;oe=6AB3A8C1; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/657150247_26426801800294267_4229617446844769500_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx2048x1536&amp;ctp=s590x590&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=5uBeSm0hyV4Q7kNvwH9eak5&amp;_nc_oc=AdqD-e9fhg29P5ptbb-bxoATLpJLzKa5ChpOU3XznPSRGg45TbRqnGiekZ-Fj2fFdn0&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=UnTMyOwTXyTerwvTKQdb8A&amp;_nc_ss=7b2a8&amp;oh=00_AQKg6QyAcUm2tguTzAJn5IZvx9Qg5619GpKKp-wmYaZQRQ&amp;oe=6AB3A834; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/654788918_26426801906960923_9152926241027148999_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx736x1000&amp;ctp=s590x590&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=4RIBSqLMeMwQ7kNvwHiyBp2&amp;_nc_oc=AdoFw7HCp0WiCNPFdtTg_qOn24YtaAUsamWcP_0v6RFoomJsna8Gnk8_8s_weRijukI&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=UnTMyOwTXyTerwvTKQdb8A&amp;_nc_ss=7b2a8&amp;oh=00_AQLX2ScQA5L21ZhRwZqfvML7zcU4HXflbHCENha7umNhbw&amp;oe=6AB3BD78; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/657400660_26426801690294278_6323538386743307505_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx736x1000&amp;ctp=s590x590&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=UVxsV1XnU1YQ7kNvwH4wdgb&amp;_nc_oc=AdoRtrvoNkiOrIL8az4oODToaK-5CuEH5v8d56ZqqHZ8_rABt700zdiT_V3Zsx3XWtI&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=UnTMyOwTXyTerwvTKQdb8A&amp;_nc_ss=7b2a8&amp;oh=00_AQK1Agtjk-e11HuLDvO8Mo64I7XyMomEEkyGgv6D6jwABQ&amp;oe=6AB399F0</t>
         </is>
       </c>
-      <c r="M12" t="n">
+      <c r="N12" t="n">
         <v>1</v>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>تنظيم وتخزين جاهز (Storage &amp; Organization)</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>rv hanging shoe organizer</t>
         </is>
       </c>
-      <c r="P12" t="n">
+      <c r="Q12" t="n">
         <v>100</v>
       </c>
-      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1257,43 +1317,44 @@
 As for laundry bag thing on wall, after testing it out this last week... ... عرض المزيد</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
         <is>
           <t>data\images\must_have_gadget_177043908\img_1.jpg; data\images\must_have_gadget_177043908\img_2.jpg; data\images\must_have_gadget_177043908\img_3.jpg; data\images\must_have_gadget_177043908\img_4.jpg; data\images\must_have_gadget_177043908\img_5.jpg</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
         <is>
           <t>Public Search</t>
         </is>
       </c>
-      <c r="J13" t="n">
+      <c r="K13" t="n">
         <v>177043908</v>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr">
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/655900116_26426801810294266_616338587343076791_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx736x1000&amp;ctp=s590x590&amp;_nc_cat=103&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=jB-xL4WCwAgQ7kNvwFsIIDC&amp;_nc_oc=AdoGV6P4nAjOyR8A4bqzpg8FsSFsTzuA9J9oYzN3nvHnZSZOlC6sXJaEQPLvrs9zuXc&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=UnTMyOwTXyTerwvTKQdb8A&amp;_nc_ss=7b2a8&amp;oh=00_AQLUYw_U16e1OluoKTx7qceTxgRUASaIWKPWYSNAPF7z1w&amp;oe=6AB3AB8A; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/656840747_26426801883627592_1775700405554872607_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx736x1000&amp;ctp=s590x590&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=j8NFBjoOyBgQ7kNvwGMUo7s&amp;_nc_oc=AdqOeMpnaO7GTgDmhNWFl03ZZ_QL7ZHss7jWCq2a7ZYSMXuKGE1WUJ9CfjqRoFvo9eU&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=UnTMyOwTXyTerwvTKQdb8A&amp;_nc_ss=7b2a8&amp;oh=00_AQJRDiTDfLxEoM8Xrvq6SX0XMQ3iNan62a_aWFxF6SNbTQ&amp;oe=6AB3A8C1; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/657150247_26426801800294267_4229617446844769500_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx2048x1536&amp;ctp=s590x590&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=5uBeSm0hyV4Q7kNvwH9eak5&amp;_nc_oc=AdqD-e9fhg29P5ptbb-bxoATLpJLzKa5ChpOU3XznPSRGg45TbRqnGiekZ-Fj2fFdn0&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=UnTMyOwTXyTerwvTKQdb8A&amp;_nc_ss=7b2a8&amp;oh=00_AQKg6QyAcUm2tguTzAJn5IZvx9Qg5619GpKKp-wmYaZQRQ&amp;oe=6AB3A834; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/654788918_26426801906960923_9152926241027148999_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx736x1000&amp;ctp=s590x590&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=4RIBSqLMeMwQ7kNvwHiyBp2&amp;_nc_oc=AdoFw7HCp0WiCNPFdtTg_qOn24YtaAUsamWcP_0v6RFoomJsna8Gnk8_8s_weRijukI&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=UnTMyOwTXyTerwvTKQdb8A&amp;_nc_ss=7b2a8&amp;oh=00_AQLX2ScQA5L21ZhRwZqfvML7zcU4HXflbHCENha7umNhbw&amp;oe=6AB3BD78; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/657400660_26426801690294278_6323538386743307505_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx736x1000&amp;ctp=s590x590&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=UVxsV1XnU1YQ7kNvwH4wdgb&amp;_nc_oc=AdoRtrvoNkiOrIL8az4oODToaK-5CuEH5v8d56ZqqHZ8_rABt700zdiT_V3Zsx3XWtI&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=UnTMyOwTXyTerwvTKQdb8A&amp;_nc_ss=7b2a8&amp;oh=00_AQK1Agtjk-e11HuLDvO8Mo64I7XyMomEEkyGgv6D6jwABQ&amp;oe=6AB399F0</t>
         </is>
       </c>
-      <c r="M13" t="n">
+      <c r="N13" t="n">
         <v>1</v>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>تنظيم وتخزين (Storage &amp; Organization)</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>rv hanging shoe organizer</t>
         </is>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>100</v>
       </c>
-      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1322,41 +1383,47 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
+          <t>Honestly didn't expect rv stabilizer x chock to work this well, but it literally solved the problem on our last trip! Best purchase I've made in a while.
+I left the direct link in the first comment for anyone who needs it 👇</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>data\images\hack_3353573731443089\img_1.jpg</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J14" t="n">
+      <c r="K14" t="n">
         <v>3353573731443089</v>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr">
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/509315519_10236268302438546_5627664025545909431_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=p526x296&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=M5yo1ydhuAIQ7kNvwFkGTxw&amp;_nc_oc=Adqlt4_mY-0WuZ0hLNgWsv01h-8e_UMZoRjTxZB7R1aPTqNOGMIVqU4-jG-oot5D2js&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQJz7r6i1K_Fsbm4nFS6qBE0tcL1ZpMwxlZa5XalCv-lgQ&amp;oe=6AB3A54C</t>
         </is>
       </c>
-      <c r="M14" t="n">
+      <c r="N14" t="n">
         <v>1</v>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>rv stabilizer x chock</t>
         </is>
       </c>
-      <c r="P14" t="n">
+      <c r="Q14" t="n">
         <v>73</v>
       </c>
-      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1385,43 +1452,50 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
+          <t>I finally stopped our camper from shaking every time the kids rolled over in their sleep.
+We tried regular jacks, but the tires were still bouncing. Locking these X-chocks between the wheels completely stopped the sway. I actually slept through the night for once!
+I left the link in the first comment 👇</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>data\images\hack_3353573731443089\img_1.jpg</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>3353573731443089</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr">
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/509315519_10236268302438546_5627664025545909431_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=p526x296&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=M5yo1ydhuAIQ7kNvwFkGTxw&amp;_nc_oc=Adqlt4_mY-0WuZ0hLNgWsv01h-8e_UMZoRjTxZB7R1aPTqNOGMIVqU4-jG-oot5D2js&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQJz7r6i1K_Fsbm4nFS6qBE0tcL1ZpMwxlZa5XalCv-lgQ&amp;oe=6AB3A54C</t>
         </is>
       </c>
-      <c r="M15" t="n">
+      <c r="N15" t="n">
         <v>1</v>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>rv stabilizer x chock</t>
         </is>
       </c>
-      <c r="P15" t="n">
+      <c r="Q15" t="n">
         <v>73</v>
       </c>
-      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1451,43 +1525,50 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
+          <t>Honest question: why do stock RV water heaters only last 90 seconds? 😅
+We used to freeze halfway through every single shower. Snagged this compact tankless heater last month and now we get endless hot water at every campsite. Total lifesaver for family trips.
+I left the link in the first comment 👇</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>data\images\must_have_gadget_3339400259527103\img_1.jpg</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr">
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>3339400259527103</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr">
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/504466196_30951392407793645_1083003521996665110_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=p526x296&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=PKBd6m8794QQ7kNvwHv6k2T&amp;_nc_oc=AdqXfd2GEhQ2tfaXL2IkQ5e03U05M1IagmAMktvw6im0SvIyX2X0BXBusblw6qbLA9Q&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=1eCUd6gOywCURufMd_fVdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQI0GDL8YgVHTfZhhbmWGQfWuXOAXKGlyQLPLfy17BdcbA&amp;oe=6AB397B0</t>
         </is>
       </c>
-      <c r="M16" t="n">
+      <c r="N16" t="n">
         <v>1</v>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>rv must have gadget</t>
         </is>
       </c>
-      <c r="P16" t="n">
+      <c r="Q16" t="n">
         <v>81</v>
       </c>
-      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1515,43 +1596,44 @@
 . We are newbies at camping. We are camping for our second time and we have hot water but it doesn't last long. We DIDNT have this switch on and the water was very hot but didn't even last one shower. Does this switch do something to make the hot water last longer? We are at a full hook up site. Coachmen Catalina legacy camper.</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
         <is>
           <t>data\images\must_have_gadget_3339400259527103\img_1.jpg</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J17" t="n">
+      <c r="K17" t="n">
         <v>3339400259527103</v>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr">
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/504466196_30951392407793645_1083003521996665110_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=p526x296&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=PKBd6m8794QQ7kNvwHv6k2T&amp;_nc_oc=AdqXfd2GEhQ2tfaXL2IkQ5e03U05M1IagmAMktvw6im0SvIyX2X0BXBusblw6qbLA9Q&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=1eCUd6gOywCURufMd_fVdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQI0GDL8YgVHTfZhhbmWGQfWuXOAXKGlyQLPLfy17BdcbA&amp;oe=6AB397B0</t>
         </is>
       </c>
-      <c r="M17" t="n">
+      <c r="N17" t="n">
         <v>1</v>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات (Gadgets &amp; Power)</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>rv must have gadget</t>
         </is>
       </c>
-      <c r="P17" t="n">
+      <c r="Q17" t="n">
         <v>81</v>
       </c>
-      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1578,39 +1660,40 @@
           <t>Has anyone ever had any luck with a manufacturers buy back on a new camper? Bought this camper right at a year ago. It’s a 2025 forest river sierra 3800rk. Purchased camper from Rocky Ridge Rv in Van Buren Arkansas (save yourself the hassle and avoid these lying fools) shortly after getting the camper we noticed it was deteriorating quickly. Things separating from the walls such as the waterfall table and our shower had a huge gap between it and the wall, camper wouldn’t leve... عرض المزيد</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
         <is>
           <t>data\images\recommendation_3845725655561225\img_1.jpg</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J18" t="n">
+      <c r="K18" t="n">
         <v>3845725655561225</v>
       </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr">
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/561728600_3814124955386211_4597581507350432745_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=p526x296&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=_H-ynFA0RAEQ7kNvwH652sw&amp;_nc_oc=AdpptTd6DXG4EzDKLZRyUHLG9uCQs_nhT9UV9cTPScoYyv5t3AObH6jdhgh-FP11MNA&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=A1RxZp9G0O8HLhEwpESXLA&amp;_nc_ss=7b2a8&amp;oh=00_AQJSpLc0DrAVWqgXHb9V1F8w2ojb5rgvV8cZ00Tsu2I1oA&amp;oe=6AB3C1B8</t>
         </is>
       </c>
-      <c r="M18" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" t="inlineStr">
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="inlineStr">
         <is>
           <t>استبعاد (نقاش/سفر/شكوى)</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1637,41 +1720,42 @@
           <t>Has anyone ever had any luck with a manufacturers buy back on a new camper? Bought this camper right at a year ago. It’s a 2025 forest river sierra 3800rk. Purchased camper from Rocky Ridge Rv in Van Buren Arkansas (save yourself the hassle and avoid these lying fools) shortly after getting the camper we noticed it was deteriorating quickly. Things separating from the walls such as the waterfall table and our shower had a huge gap between it and the wall, camper wouldn’t leve... عرض المزيد</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
         <is>
           <t>data\images\recommendation_3845725655561225\img_1.jpg</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>3845725655561225</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr">
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/561728600_3814124955386211_4597581507350432745_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=p526x296&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=_H-ynFA0RAEQ7kNvwH652sw&amp;_nc_oc=AdpptTd6DXG4EzDKLZRyUHLG9uCQs_nhT9UV9cTPScoYyv5t3AObH6jdhgh-FP11MNA&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=A1RxZp9G0O8HLhEwpESXLA&amp;_nc_ss=7b2a8&amp;oh=00_AQJSpLc0DrAVWqgXHb9V1F8w2ojb5rgvV8cZ00Tsu2I1oA&amp;oe=6AB3C1B8</t>
         </is>
       </c>
-      <c r="M19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" t="inlineStr">
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="inlineStr">
         <is>
           <t>استبعاد (نقاش/سفر/شكوى)</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1700,43 +1784,49 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
+          <t>Honestly didn't expect rv amazon find to work this well, but it literally solved the problem on our last trip! Best purchase I've made in a while.
+I left the direct link in the first comment for anyone who needs it 👇</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
           <t>data\images\amazon_find_791791057\img_1.jpg; data\images\amazon_find_791791057\img_2.jpg; data\images\amazon_find_791791057\img_3.jpg; data\images\amazon_find_791791057\img_4.jpg</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
         <is>
           <t>Public Search</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>791791057</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr">
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/718204993_3377270389114032_3017451080494617445_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx2048x1536&amp;ctp=s590x590&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=qYfYw4OVFlQQ7kNvwFzTUw2&amp;_nc_oc=AdrTdokM1V_C9TzLfjq5_yhdW9z1pnNrXAPOqM7sMo9zBm1IgAoSMyik8zLi5QctYCQ&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=MKX-JBaFHpnqnEGtSRwW4A&amp;_nc_ss=7b2a8&amp;oh=00_AQKN6mRZQV1JOvOk5cGH3-J9bLpZnNAF30D41_tiHhRwqA&amp;oe=6AB393CE; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/719160410_3377257819115289_4512916211874135718_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx960x720&amp;ctp=s590x590&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=kme4VsbYGiQQ7kNvwF0UTnh&amp;_nc_oc=AdpLFsFTOQlfY2GtWNtHZkgfNauVxu3L28i1m9bTX7UjZW46L_6uJXsumd63ry3hM_E&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=MKX-JBaFHpnqnEGtSRwW4A&amp;_nc_ss=7b2a8&amp;oh=00_AQIpFVodpDrLXaNrm03MWNxcRUQTUe0bD15QwfGTs15G_A&amp;oe=6AB39474; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/715749899_3377270385780699_46444169963824531_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=s590x590&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=m1B9Z9a3XTcQ7kNvwHbSueQ&amp;_nc_oc=AdqZvLfkUECCp-PzosWPpwH6aKcCTcnp5LCTlPaQnAapvNYk3h0vr0MwYZ74N6JJE60&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=MKX-JBaFHpnqnEGtSRwW4A&amp;_nc_ss=7b2a8&amp;oh=00_AQIIaHm-ZLLeWqyzE87P30_-cNCHO9sQVloN5bT3aFotpg&amp;oe=6AB395EC; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/720495745_3377270445780693_888169211609445957_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=s590x590&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=PEd1aWG90c4Q7kNvwFfUOQ4&amp;_nc_oc=AdrTRXfrx1pomRzcompzkQAMeyuhMDOb6GxUxdzedExILCEZNRNmCOswHKYdYi-vFpY&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=MKX-JBaFHpnqnEGtSRwW4A&amp;_nc_ss=7b2a8&amp;oh=00_AQJdSmbYZUx1bo6s6BUqTCImTGV2rJasH5LeKQDXXFya1A&amp;oe=6AB3A127</t>
         </is>
       </c>
-      <c r="M20" t="n">
+      <c r="N20" t="n">
         <v>1</v>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="P20" t="inlineStr">
         <is>
           <t>rv amazon find</t>
         </is>
       </c>
-      <c r="P20" t="n">
+      <c r="Q20" t="n">
         <v>83</v>
       </c>
-      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1763,43 +1853,44 @@
           <t>You guys were so helpful when I asked for advice so I thought I’d share a few of my “hacks” to maybe help someone else! ... عرض المزيد</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
         <is>
           <t>data\images\amazon_find_791791057\img_1.jpg; data\images\amazon_find_791791057\img_2.jpg; data\images\amazon_find_791791057\img_3.jpg; data\images\amazon_find_791791057\img_4.jpg</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
         <is>
           <t>Public Search</t>
         </is>
       </c>
-      <c r="J21" t="n">
+      <c r="K21" t="n">
         <v>791791057</v>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr">
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/718204993_3377270389114032_3017451080494617445_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx2048x1536&amp;ctp=s590x590&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=qYfYw4OVFlQQ7kNvwFzTUw2&amp;_nc_oc=AdrTdokM1V_C9TzLfjq5_yhdW9z1pnNrXAPOqM7sMo9zBm1IgAoSMyik8zLi5QctYCQ&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=MKX-JBaFHpnqnEGtSRwW4A&amp;_nc_ss=7b2a8&amp;oh=00_AQKN6mRZQV1JOvOk5cGH3-J9bLpZnNAF30D41_tiHhRwqA&amp;oe=6AB393CE; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/719160410_3377257819115289_4512916211874135718_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx960x720&amp;ctp=s590x590&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=kme4VsbYGiQQ7kNvwF0UTnh&amp;_nc_oc=AdpLFsFTOQlfY2GtWNtHZkgfNauVxu3L28i1m9bTX7UjZW46L_6uJXsumd63ry3hM_E&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=MKX-JBaFHpnqnEGtSRwW4A&amp;_nc_ss=7b2a8&amp;oh=00_AQIpFVodpDrLXaNrm03MWNxcRUQTUe0bD15QwfGTs15G_A&amp;oe=6AB39474; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/715749899_3377270385780699_46444169963824531_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=s590x590&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=m1B9Z9a3XTcQ7kNvwHbSueQ&amp;_nc_oc=AdqZvLfkUECCp-PzosWPpwH6aKcCTcnp5LCTlPaQnAapvNYk3h0vr0MwYZ74N6JJE60&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=MKX-JBaFHpnqnEGtSRwW4A&amp;_nc_ss=7b2a8&amp;oh=00_AQIIaHm-ZLLeWqyzE87P30_-cNCHO9sQVloN5bT3aFotpg&amp;oe=6AB395EC; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/720495745_3377270445780693_888169211609445957_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=s590x590&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=PEd1aWG90c4Q7kNvwFfUOQ4&amp;_nc_oc=AdrTRXfrx1pomRzcompzkQAMeyuhMDOb6GxUxdzedExILCEZNRNmCOswHKYdYi-vFpY&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=MKX-JBaFHpnqnEGtSRwW4A&amp;_nc_ss=7b2a8&amp;oh=00_AQJdSmbYZUx1bo6s6BUqTCImTGV2rJasH5LeKQDXXFya1A&amp;oe=6AB3A127</t>
         </is>
       </c>
-      <c r="M21" t="n">
+      <c r="N21" t="n">
         <v>1</v>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>إكسسوارات وحلول ذكية (Smart Accessories &amp; Hacks)</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="P21" t="inlineStr">
         <is>
           <t>rv amazon find</t>
         </is>
       </c>
-      <c r="P21" t="n">
+      <c r="Q21" t="n">
         <v>91</v>
       </c>
-      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1829,41 +1920,47 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
+          <t>Honestly didn't expect rv stabilizer x chock to work this well, but it literally solved the problem on our last trip! Best purchase I've made in a while.
+I left the direct link in the first comment for anyone who needs it 👇</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
           <t>data\images\hack_3583318008493819\img_1.jpg; data\images\hack_3583318008493819\img_2.jpg; data\images\hack_3583318008493819\img_3.jpg</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J22" t="n">
+      <c r="K22" t="n">
         <v>3583318008493819</v>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr">
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/763072132_10240527915834058_262860686266165320_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1152x2048&amp;ctp=s590x590&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=tQPKb_7z3scQ7kNvwHI1W7g&amp;_nc_oc=AdryOCOHLUetXqxLh_YB0dln50lhK5trI90T_Fm1qocc_zcSjKjM7rFYwajXvgsjhTI&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=ViAqpShX1Nm9L2g-4A-cEw&amp;_nc_ss=7b2a8&amp;oh=00_AQJ0GnPf57poAwnS1tveFqIifG41xCwgcTXoj7nwXsPD0g&amp;oe=6AB39330; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/764719882_10240527916554076_6179174592261675065_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1152x2048&amp;ctp=s590x590&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=DGePznIup-IQ7kNvwF8n1gs&amp;_nc_oc=AdpGktVoydqk0AxdQDAOzbx_Pf2MDjo3DIQObD1Zjm6Y7VQBbann44VUTt2JZv16NT8&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=ViAqpShX1Nm9L2g-4A-cEw&amp;_nc_ss=7b2a8&amp;oh=00_AQJvlQLTekeLpX0VeuXsY7AW8BTlFEb4ontl07T28WmncA&amp;oe=6AB39768; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/762276276_10240527918834133_6935526286052437077_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1152x2048&amp;ctp=s590x590&amp;_nc_cat=104&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=LUYt4ZPtFlQQ7kNvwFtDGTf&amp;_nc_oc=Ados7w7e5WTUF89zeazhrONFUSOjfR3KkU-WEt4FzNzv3RCM9gJpPLl89FV5RIzy0P4&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=ViAqpShX1Nm9L2g-4A-cEw&amp;_nc_ss=7b2a8&amp;oh=00_AQIUbRAOYKraspj5sBL0vF-0I_3MUiK5eLiusqFF-B6VQQ&amp;oe=6AB3908B</t>
         </is>
       </c>
-      <c r="M22" t="n">
+      <c r="N22" t="n">
         <v>1</v>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="P22" t="inlineStr">
         <is>
           <t>rv stabilizer x chock</t>
         </is>
       </c>
-      <c r="P22" t="n">
+      <c r="Q22" t="n">
         <v>83</v>
       </c>
-      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1893,43 +1990,50 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
+          <t>If your RV rocks every time someone takes a single step inside, you need to try this.
+Our rig was perfectly level, but the floor still shook constantly. We tossed a set of X-chocks between the tires and it instantly locked everything solid. Worth every penny!
+I left the link in the first comment if you want to grab a pair 👇</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
           <t>data\images\hack_3583318008493819\img_1.jpg; data\images\hack_3583318008493819\img_2.jpg; data\images\hack_3583318008493819\img_3.jpg</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr">
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>3583318008493819</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr">
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/763072132_10240527915834058_262860686266165320_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1152x2048&amp;ctp=s590x590&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=tQPKb_7z3scQ7kNvwHI1W7g&amp;_nc_oc=AdryOCOHLUetXqxLh_YB0dln50lhK5trI90T_Fm1qocc_zcSjKjM7rFYwajXvgsjhTI&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=ViAqpShX1Nm9L2g-4A-cEw&amp;_nc_ss=7b2a8&amp;oh=00_AQJ0GnPf57poAwnS1tveFqIifG41xCwgcTXoj7nwXsPD0g&amp;oe=6AB39330; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/764719882_10240527916554076_6179174592261675065_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1152x2048&amp;ctp=s590x590&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=DGePznIup-IQ7kNvwF8n1gs&amp;_nc_oc=AdpGktVoydqk0AxdQDAOzbx_Pf2MDjo3DIQObD1Zjm6Y7VQBbann44VUTt2JZv16NT8&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=ViAqpShX1Nm9L2g-4A-cEw&amp;_nc_ss=7b2a8&amp;oh=00_AQJvlQLTekeLpX0VeuXsY7AW8BTlFEb4ontl07T28WmncA&amp;oe=6AB39768; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/762276276_10240527918834133_6935526286052437077_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1152x2048&amp;ctp=s590x590&amp;_nc_cat=104&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=LUYt4ZPtFlQQ7kNvwFtDGTf&amp;_nc_oc=Ados7w7e5WTUF89zeazhrONFUSOjfR3KkU-WEt4FzNzv3RCM9gJpPLl89FV5RIzy0P4&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=ViAqpShX1Nm9L2g-4A-cEw&amp;_nc_ss=7b2a8&amp;oh=00_AQIUbRAOYKraspj5sBL0vF-0I_3MUiK5eLiusqFF-B6VQQ&amp;oe=6AB3908B</t>
         </is>
       </c>
-      <c r="M23" t="n">
+      <c r="N23" t="n">
         <v>1</v>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="P23" t="inlineStr">
         <is>
           <t>rv stabilizer x chock</t>
         </is>
       </c>
-      <c r="P23" t="n">
+      <c r="Q23" t="n">
         <v>83</v>
       </c>
-      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1956,41 +2060,42 @@
           <t>Hi all my husband and I bought our first ever brand new 2021 hideout! With one slideout! We bought it in April of this year! We were loving it so much, it was my dream ... عرض المزيد</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
         <is>
           <t>data\images\must_have_gadget_2519590198174784\img_1.jpg</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr">
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>2519590198174784</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr">
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/489965465_10161600930962880_4833098666534324521_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1504x2015&amp;ctp=p526x296&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=536f4a&amp;_nc_ohc=xMIVUG5htDkQ7kNvwG8ehE-&amp;_nc_oc=Adp4sJx_jBWQxqAezLmKNS9_5TDHX2yXRWxyb3DDrZ3-anVVRKHC96Jtv_1gNntBUhE&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=xdIPSj7R-3lhEMKdb3QlGQ&amp;_nc_ss=7b2a8&amp;oh=00_AQKdYBPNRTeYp1FOp6-rBTffCUwYr55-PcsfEHer1NRGrw&amp;oe=6AB3994F</t>
         </is>
       </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="inlineStr">
+      <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="inlineStr">
         <is>
           <t>استبعاد (نقاش/سفر/شكوى)</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2017,43 +2122,44 @@
           <t>Hi all my husband and I bought our first ever brand new 2021 hideout! With one slideout! We bought it in April of this year! We were loving it so much, it was my dream ... عرض المزيد</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
         <is>
           <t>data\images\must_have_gadget_2519590198174784\img_1.jpg</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J25" t="n">
+      <c r="K25" t="n">
         <v>2519590198174784</v>
       </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr">
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/489965465_10161600930962880_4833098666534324521_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1504x2015&amp;ctp=p526x296&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=536f4a&amp;_nc_ohc=xMIVUG5htDkQ7kNvwG8ehE-&amp;_nc_oc=Adp4sJx_jBWQxqAezLmKNS9_5TDHX2yXRWxyb3DDrZ3-anVVRKHC96Jtv_1gNntBUhE&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=xdIPSj7R-3lhEMKdb3QlGQ&amp;_nc_ss=7b2a8&amp;oh=00_AQKdYBPNRTeYp1FOp6-rBTffCUwYr55-PcsfEHer1NRGrw&amp;oe=6AB3994F</t>
         </is>
       </c>
-      <c r="M25" t="n">
+      <c r="N25" t="n">
         <v>1</v>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات (Gadgets &amp; Power)</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
+      <c r="P25" t="inlineStr">
         <is>
           <t>rv must have gadget</t>
         </is>
       </c>
-      <c r="P25" t="n">
+      <c r="Q25" t="n">
         <v>89</v>
       </c>
-      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2086,41 +2192,47 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
+          <t>Honestly didn't expect rv small dehumidifier to work this well, but it literally solved the problem on our last trip! Best purchase I've made in a while.
+I left the direct link in the first comment for anyone who needs it 👇</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
           <t>data\images\hack_3513687305456890\img_1.jpg; data\images\hack_3513687305456890\img_2.jpg</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J26" t="n">
+      <c r="K26" t="n">
         <v>3513687305456890</v>
       </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr">
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/711643338_4031111337187636_2883491981945560264_n.jpg?stp=cp6_dst-jpegr_tt6&amp;cstp=mx2048x1536&amp;ctp=s590x590&amp;_nc_cat=101&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=f_dNgnnJOYgQ7kNvwExjlSF&amp;_nc_oc=AdrWkULW0up9vpUlFyOdOOVFswpvqlDIhNLfoyhWvHBlMRRjGZi30e5xunQe5kh6Z0Q&amp;_nc_zt=23&amp;se=-1&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=ViAqpShX1Nm9L2g-4A-cEw&amp;_nc_ss=7b2a8&amp;oh=00_AQKTSnMNFsMvYlBm6Q9Cs_j26ctmUP0uKKMt38ogPK1CCQ&amp;oe=6AB3BE3A; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/710079281_4031111510520952_7622572342432142030_n.jpg?stp=cp6_dst-jpegr_tt6&amp;cstp=mx1536x2048&amp;ctp=s590x590&amp;_nc_cat=104&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=4dRi6V0TjK4Q7kNvwHSnOiX&amp;_nc_oc=AdrDAS7dm4zU-dcnhVK6W-knhBbh3pssG6jJndvEsBOKEvFfAFNNPsyLOvKMWjs_ivI&amp;_nc_zt=23&amp;se=-1&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=ViAqpShX1Nm9L2g-4A-cEw&amp;_nc_ss=7b2a8&amp;oh=00_AQI6pqkPWZ9WIOjSIkSrF2puVgdYZN4nCE9eR76sArCmFA&amp;oe=6AB3B093</t>
         </is>
       </c>
-      <c r="M26" t="n">
+      <c r="N26" t="n">
         <v>1</v>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
+      <c r="P26" t="inlineStr">
         <is>
           <t>rv small dehumidifier</t>
         </is>
       </c>
-      <c r="P26" t="n">
+      <c r="Q26" t="n">
         <v>70</v>
       </c>
-      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2153,43 +2265,49 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
+          <t>Honestly didn't expect rv small dehumidifier to work this well, but it literally solved the problem on our last trip! Best purchase I've made in a while.
+I left the direct link in the first comment for anyone who needs it 👇</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
           <t>data\images\hack_3513687305456890\img_1.jpg; data\images\hack_3513687305456890\img_2.jpg</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr">
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>3513687305456890</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr">
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/711643338_4031111337187636_2883491981945560264_n.jpg?stp=cp6_dst-jpegr_tt6&amp;cstp=mx2048x1536&amp;ctp=s590x590&amp;_nc_cat=101&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=f_dNgnnJOYgQ7kNvwExjlSF&amp;_nc_oc=AdrWkULW0up9vpUlFyOdOOVFswpvqlDIhNLfoyhWvHBlMRRjGZi30e5xunQe5kh6Z0Q&amp;_nc_zt=23&amp;se=-1&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=ViAqpShX1Nm9L2g-4A-cEw&amp;_nc_ss=7b2a8&amp;oh=00_AQKTSnMNFsMvYlBm6Q9Cs_j26ctmUP0uKKMt38ogPK1CCQ&amp;oe=6AB3BE3A; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/710079281_4031111510520952_7622572342432142030_n.jpg?stp=cp6_dst-jpegr_tt6&amp;cstp=mx1536x2048&amp;ctp=s590x590&amp;_nc_cat=104&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=4dRi6V0TjK4Q7kNvwHSnOiX&amp;_nc_oc=AdrDAS7dm4zU-dcnhVK6W-knhBbh3pssG6jJndvEsBOKEvFfAFNNPsyLOvKMWjs_ivI&amp;_nc_zt=23&amp;se=-1&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=ViAqpShX1Nm9L2g-4A-cEw&amp;_nc_ss=7b2a8&amp;oh=00_AQI6pqkPWZ9WIOjSIkSrF2puVgdYZN4nCE9eR76sArCmFA&amp;oe=6AB3B093</t>
         </is>
       </c>
-      <c r="M27" t="n">
+      <c r="N27" t="n">
         <v>1</v>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="P27" t="inlineStr">
         <is>
           <t>rv small dehumidifier</t>
         </is>
       </c>
-      <c r="P27" t="n">
+      <c r="Q27" t="n">
         <v>70</v>
       </c>
-      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2221,43 +2339,51 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
+          <t>Almost had a heart attack when my toddler opened our RV door in the middle of the night.
+Standard locks weren't cutting it, but this cheap Amazon safety lock mounts up high with zero drilling required.
+Now I can actually sleep soundly on our trips! 
+I left the link in the first comment 👇</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
           <t>data\images\amazon_find_2956335967833536\img_1.jpg</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>2956335967833536</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr">
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/486263063_3431305033666747_2774947844339664550_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=p526x296&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=_V3lAOuS71gQ7kNvwG1HA6t&amp;_nc_oc=Ado0M-qFkVhQnVlLURz25aP5SNH_jAdpe4Dmc4HtVTUByPMy0vPdcFtq1ganZeRHiEc&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=-DNXGqSwxAYHz3InfHrB2g&amp;_nc_ss=7b2a8&amp;oh=00_AQK8ZOwXZcwYIiJ5OsCjs7fTQm9bTUEleRwYHx_4DZJBiw&amp;oe=6AB39B39</t>
         </is>
       </c>
-      <c r="M28" t="n">
+      <c r="N28" t="n">
         <v>1</v>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t>إكسسوارات وأدوات تجارية (Commercial Gear &amp; Accessories)</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="P28" t="inlineStr">
         <is>
           <t>rv amazon find</t>
         </is>
       </c>
-      <c r="P28" t="n">
+      <c r="Q28" t="n">
         <v>81</v>
       </c>
-      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2287,43 +2413,44 @@
 Any suggestions on good locks? ... عرض المزيد</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
         <is>
           <t>data\images\amazon_find_2956335967833536\img_1.jpg</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr">
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J29" t="n">
+      <c r="K29" t="n">
         <v>2956335967833536</v>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr">
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/486263063_3431305033666747_2774947844339664550_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=p526x296&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=_V3lAOuS71gQ7kNvwG1HA6t&amp;_nc_oc=Ado0M-qFkVhQnVlLURz25aP5SNH_jAdpe4Dmc4HtVTUByPMy0vPdcFtq1ganZeRHiEc&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=-DNXGqSwxAYHz3InfHrB2g&amp;_nc_ss=7b2a8&amp;oh=00_AQK8ZOwXZcwYIiJ5OsCjs7fTQm9bTUEleRwYHx_4DZJBiw&amp;oe=6AB39B39</t>
         </is>
       </c>
-      <c r="M29" t="n">
+      <c r="N29" t="n">
         <v>1</v>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t>إكسسوارات وحلول ذكية (Smart Accessories &amp; Hacks)</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="P29" t="inlineStr">
         <is>
           <t>rv amazon find</t>
         </is>
       </c>
-      <c r="P29" t="n">
+      <c r="Q29" t="n">
         <v>81</v>
       </c>
-      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2351,39 +2478,40 @@
 On our first trip, the slide out wouldn’t retract all the way on its own (yes, I checked it prior to purchase and it seemed to work fine, but looking back, I think they had it jacked up on that side to help assist it and I just thought the driveway was pitched). It would get about a foot out and come to a stop. If I had it jacked up slightly and leaned into it, I ... عرض المزيد</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
         <is>
           <t>data\images\recommendation_4219763604824093\img_1.jpg</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr">
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J30" t="n">
+      <c r="K30" t="n">
         <v>4219763604824093</v>
       </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr">
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/778928638_10234377270479258_6720371812830267357_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1206x773&amp;ctp=p180x540&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=2MFpcUQX5nAQ7kNvwGeefCS&amp;_nc_oc=AdpY7NG2vbXAeZdlBhdLZ0XnO1G2KpbNq-q-Vi50uubkYztx7ASFIj4MVK_Shql8qB8&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=A8Me3j8jNja1Mkq3I5rYPg&amp;_nc_ss=7b2a8&amp;oh=00_AQJ-yYB_jczpZmho-tcYD7J0ValNk1dW5sFyRVmDscJnXQ&amp;oe=6AB396CA</t>
         </is>
       </c>
-      <c r="M30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" t="inlineStr">
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="inlineStr">
         <is>
           <t>استبعاد (نقاش/سفر/شكوى)</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2411,41 +2539,42 @@
 On our first trip, the slide out wouldn’t retract all the way on its own (yes, I checked it prior to purchase and it seemed to work fine, but looking back, I think they had it jacked up on that side to help assist it and I just thought the driveway was pitched). It would get about a foot out and come to a stop. If I had it jacked up slightly and leaned into it, I ... عرض المزيد</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
         <is>
           <t>data\images\recommendation_4219763604824093\img_1.jpg</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr">
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>4219763604824093</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr">
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/778928638_10234377270479258_6720371812830267357_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1206x773&amp;ctp=p180x540&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=2MFpcUQX5nAQ7kNvwGeefCS&amp;_nc_oc=AdpY7NG2vbXAeZdlBhdLZ0XnO1G2KpbNq-q-Vi50uubkYztx7ASFIj4MVK_Shql8qB8&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=A8Me3j8jNja1Mkq3I5rYPg&amp;_nc_ss=7b2a8&amp;oh=00_AQJ-yYB_jczpZmho-tcYD7J0ValNk1dW5sFyRVmDscJnXQ&amp;oe=6AB396CA</t>
         </is>
       </c>
-      <c r="M31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" t="inlineStr">
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="inlineStr">
         <is>
           <t>استبعاد (نقاش/سفر/شكوى)</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2474,43 +2603,51 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
+          <t>If your stinky slinky won’t fit inside your RV bumper, stop forcing it. 
+I got tired of wrestling mine and grabbed this under-rig storage tube on Amazon. 
+Fits the thick fittings easily and mounts right to the frame in 10 minutes. 
+Left the link in the comments if you need one! 👇</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
           <t>data\images\amazon_find_4228244110642709\img_1.jpg</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr">
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>4228244110642709</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr">
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/789447152_10244813111573647_47739271540443468_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx720x1280&amp;ctp=p526x296&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=9RQ21jppgcUQ7kNvwHOPHq-&amp;_nc_oc=AdpS_m5-K5_RU2sUwoQJWJrY-sl4KHrcU30zbIzSrUQ3R25NJhL2uHJx88ZWQYW0umU&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=-DNXGqSwxAYHz3InfHrB2g&amp;_nc_ss=7b2a8&amp;oh=00_AQKmJVCGhzzaIOrLJSB17QoEwCChxJioCHSDOxuyqiFvMA&amp;oe=6AB3A606</t>
         </is>
       </c>
-      <c r="M32" t="n">
+      <c r="N32" t="n">
         <v>1</v>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>تنظيم وتخزين جاهز (Storage &amp; Organization)</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
+      <c r="P32" t="inlineStr">
         <is>
           <t>rv amazon find</t>
         </is>
       </c>
-      <c r="P32" t="n">
+      <c r="Q32" t="n">
         <v>81</v>
       </c>
-      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2537,43 +2674,44 @@
           <t>My stinky slinky won’t fit in the bumper tubing. Any ideas?</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
         <is>
           <t>data\images\amazon_find_4228244110642709\img_1.jpg</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr">
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J33" t="n">
+      <c r="K33" t="n">
         <v>4228244110642709</v>
       </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr">
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/789447152_10244813111573647_47739271540443468_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx720x1280&amp;ctp=p526x296&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=9RQ21jppgcUQ7kNvwHOPHq-&amp;_nc_oc=AdpS_m5-K5_RU2sUwoQJWJrY-sl4KHrcU30zbIzSrUQ3R25NJhL2uHJx88ZWQYW0umU&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=-DNXGqSwxAYHz3InfHrB2g&amp;_nc_ss=7b2a8&amp;oh=00_AQKmJVCGhzzaIOrLJSB17QoEwCChxJioCHSDOxuyqiFvMA&amp;oe=6AB3A606</t>
         </is>
       </c>
-      <c r="M33" t="n">
+      <c r="N33" t="n">
         <v>1</v>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="O33" t="inlineStr">
         <is>
           <t>تنظيم وتخزين (Storage &amp; Organization)</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
+      <c r="P33" t="inlineStr">
         <is>
           <t>rv amazon find</t>
         </is>
       </c>
-      <c r="P33" t="n">
+      <c r="Q33" t="n">
         <v>81</v>
       </c>
-      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2600,41 +2738,42 @@
           <t>Soo I want to paint the walls in my camper and I was wondering is there a certain paint or way to go about doing this? Below is what my walls look like in my camper.</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
         <is>
           <t>data\images\must_have_gadget_3605957036204756\img_1.jpg</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr">
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>3605957036204756</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr">
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/514417036_24232386396387276_8898425086872934580_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=p526x296&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=0WuEyVKJSqkQ7kNvwGxzTrJ&amp;_nc_oc=AdpwYEulmgEEsjJgMkkuOg0h0LPQX5Bi_s7roUkZ1JKXJsLZhWL2MrHLy_UyPk1-mPA&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=xdIPSj7R-3lhEMKdb3QlGQ&amp;_nc_ss=7b2a8&amp;oh=00_AQKl3JPpvV7FsczmsCXiMGk3JcjuvjpM0ztQZBAozZpITg&amp;oe=6AB3CB59</t>
         </is>
       </c>
-      <c r="M34" t="n">
-        <v>0</v>
-      </c>
-      <c r="N34" t="inlineStr">
+      <c r="N34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" t="inlineStr">
         <is>
           <t>استبعاد (نقاش/سفر/شكوى)</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2661,43 +2800,44 @@
           <t>Soo I want to paint the walls in my camper and I was wondering is there a certain paint or way to go about doing this? Below is what my walls look like in my camper.</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
         <is>
           <t>data\images\must_have_gadget_3605957036204756\img_1.jpg</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr">
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J35" t="n">
+      <c r="K35" t="n">
         <v>3605957036204756</v>
       </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr">
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/514417036_24232386396387276_8898425086872934580_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=p526x296&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=0WuEyVKJSqkQ7kNvwGxzTrJ&amp;_nc_oc=AdpwYEulmgEEsjJgMkkuOg0h0LPQX5Bi_s7roUkZ1JKXJsLZhWL2MrHLy_UyPk1-mPA&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=xdIPSj7R-3lhEMKdb3QlGQ&amp;_nc_ss=7b2a8&amp;oh=00_AQKl3JPpvV7FsczmsCXiMGk3JcjuvjpM0ztQZBAozZpITg&amp;oe=6AB3CB59</t>
         </is>
       </c>
-      <c r="M35" t="n">
+      <c r="N35" t="n">
         <v>1</v>
       </c>
-      <c r="N35" t="inlineStr">
+      <c r="O35" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات (Gadgets &amp; Power)</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
+      <c r="P35" t="inlineStr">
         <is>
           <t>rv must have gadget</t>
         </is>
       </c>
-      <c r="P35" t="n">
+      <c r="Q35" t="n">
         <v>81</v>
       </c>
-      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2726,29 +2866,30 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr">
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J36" t="n">
+      <c r="K36" t="n">
         <v>4242996285834158</v>
       </c>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
-      <c r="M36" t="n">
-        <v>0</v>
-      </c>
-      <c r="N36" t="inlineStr">
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2777,31 +2918,32 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr">
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>4242996285834158</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
-      <c r="M37" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" t="inlineStr">
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2830,31 +2972,32 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr">
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>3581840501974903</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
-      <c r="M38" t="n">
-        <v>0</v>
-      </c>
-      <c r="N38" t="inlineStr">
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="n">
+        <v>0</v>
+      </c>
+      <c r="R38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2883,21 +3026,22 @@
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr">
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J39" t="n">
+      <c r="K39" t="n">
         <v>3581840501974903</v>
       </c>
-      <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2926,29 +3070,30 @@
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr">
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J40" t="n">
+      <c r="K40" t="n">
         <v>4244102009056919</v>
       </c>
-      <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
-      <c r="M40" t="n">
-        <v>0</v>
-      </c>
-      <c r="N40" t="inlineStr">
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2977,31 +3122,32 @@
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr">
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>4244102009056919</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
-      <c r="M41" t="n">
-        <v>0</v>
-      </c>
-      <c r="N41" t="inlineStr">
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3030,31 +3176,32 @@
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr">
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>3622362671256019</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
-      <c r="M42" t="n">
-        <v>0</v>
-      </c>
-      <c r="N42" t="inlineStr">
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="n">
+        <v>0</v>
+      </c>
+      <c r="R42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3083,21 +3230,22 @@
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr">
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J43" t="n">
+      <c r="K43" t="n">
         <v>3622362671256019</v>
       </c>
-      <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3124,39 +3272,40 @@
           <t>My motor home is five years old and the fiberglass is getting a little dull. I would appreciate recommendations for a product that will remove the oxidation, give it some shine, and not damage the vinyl graphics. Preferably a product that will be kind to 72 year old shoulders and not break the bank. Am I asking too much?</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
         <is>
           <t>data\images\recommendation_3628769393948680\img_1.jpg</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr">
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J44" t="n">
+      <c r="K44" t="n">
         <v>3628769393948680</v>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr">
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/808052775_10215713116376802_6417467035183016827_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx2048x1536&amp;ctp=s720x720&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=5aeIRrCJGp4Q7kNvwHvDyKy&amp;_nc_oc=AdqG_YVwrxVe6Fyw0hKRqTYuhf09LUF3aWqDHRgNV4bC3Ywaab_Alz2SaleHUdgWCOA&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=vfknkuq86QfA8Lw-aBT1Xw&amp;_nc_ss=7b2a8&amp;oh=00_AQKVtcAXNMkkVDiI2ToSgwRqlB1V4TAv598oTL1uJTj_nw&amp;oe=6AB3A6DD</t>
         </is>
       </c>
-      <c r="M44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N44" t="inlineStr">
+      <c r="N44" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" t="inlineStr">
         <is>
           <t>غير مؤكد (نقاش عام)</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="n">
+        <v>0</v>
+      </c>
+      <c r="R44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3183,41 +3332,42 @@
           <t>My motor home is five years old and the fiberglass is getting a little dull. I would appreciate recommendations for a product that will remove the oxidation, give it some shine, and not damage the vinyl graphics. Preferably a product that will be kind to 72 year old shoulders and not break the bank. Am I asking too much?</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
         <is>
           <t>data\images\recommendation_3628769393948680\img_1.jpg</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr">
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>3628769393948680</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr">
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/808052775_10215713116376802_6417467035183016827_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx2048x1536&amp;ctp=s720x720&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=5aeIRrCJGp4Q7kNvwHvDyKy&amp;_nc_oc=AdqG_YVwrxVe6Fyw0hKRqTYuhf09LUF3aWqDHRgNV4bC3Ywaab_Alz2SaleHUdgWCOA&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=vfknkuq86QfA8Lw-aBT1Xw&amp;_nc_ss=7b2a8&amp;oh=00_AQKVtcAXNMkkVDiI2ToSgwRqlB1V4TAv598oTL1uJTj_nw&amp;oe=6AB3A6DD</t>
         </is>
       </c>
-      <c r="M45" t="n">
-        <v>0</v>
-      </c>
-      <c r="N45" t="inlineStr">
+      <c r="N45" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" t="inlineStr">
         <is>
           <t>غير مؤكد (نقاش عام)</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3247,31 +3397,32 @@
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr">
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>3218284608305336</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
-      <c r="M46" t="n">
-        <v>0</v>
-      </c>
-      <c r="N46" t="inlineStr">
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="n">
+        <v>0</v>
+      </c>
+      <c r="R46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3301,143 +3452,151 @@
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr">
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J47" t="n">
+      <c r="K47" t="n">
         <v>3218284608305336</v>
       </c>
-      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
-      <c r="M47" t="n">
-        <v>0</v>
-      </c>
-      <c r="N47" t="inlineStr">
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="n">
+        <v>0</v>
+      </c>
+      <c r="R47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>recommendation</t>
+          <t>amazon find</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>8</v>
       </c>
       <c r="C48" t="n">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="D48" t="n">
         <v>0</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/roadtreking/posts/3359003754258580/</t>
+          <t>https://www.facebook.com/groups/RVhackcamp/posts/4147910648676056/</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Looking for recommendation on the best route (east to west) through Dallas /Ft Worth.   Midweek, hitting Dallas around Noon.  Pulling 36ft 5th wheel</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>roadtreking</t>
-        </is>
-      </c>
-      <c r="J48" t="n">
-        <v>3359003754258580</v>
-      </c>
-      <c r="K48" t="inlineStr"/>
+          <t>Does anyone have a hack for cooling the bottom bunk better? We’ve tried mini fans but they don’t seem to stay upright or stick to the walls very well. I wish we could get an ac vent in there!</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Honestly didn't expect rv 12v portable bunk fan to work this well, but it literally solved the problem on our last trip! Best purchase I've made in a while.
+I left the direct link in the first comment for anyone who needs it 👇</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>data\images\amazon_find_4147910648676056\img_1.jpg</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>RVhackcamp</t>
+        </is>
+      </c>
+      <c r="K48" t="n">
+        <v>4147910648676056</v>
+      </c>
       <c r="L48" t="inlineStr"/>
-      <c r="M48" t="n">
-        <v>0</v>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>غير مؤهل (بدون صور)</t>
-        </is>
-      </c>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/730771479_10102373262656439_2111230534189182674_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1206x952&amp;ctp=s640x640&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=DGSaV9gAmTAQ7kNvwEywMS_&amp;_nc_oc=AdprvPdL0g_5W2xgZVeuTA___ucidu0kEo0UPwtfNjLrGr8lzJOIt34RmN_8IoOdX94&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=-DNXGqSwxAYHz3InfHrB2g&amp;_nc_ss=7b2a8&amp;oh=00_AQKuI7NhSiWUW3pweIYcuSccGm2fBiXhQmnukqpjQKDiRg&amp;oe=6AB3C7D6</t>
+        </is>
+      </c>
+      <c r="N48" t="n">
+        <v>1</v>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>rv 12v portable bunk fan</t>
+        </is>
+      </c>
+      <c r="Q48" t="n">
+        <v>81</v>
+      </c>
+      <c r="R48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>hack</t>
+          <t>recommendation</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>8</v>
       </c>
       <c r="C49" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="D49" t="n">
         <v>0</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/RVhackcamp/posts/4147910648676056/</t>
+          <t>https://www.facebook.com/groups/roadtreking/posts/3359003754258580/</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Does anyone have a hack for cooling the bottom bunk better? We’ve tried mini fans but they don’t seem to stay upright or stick to the walls very well. I wish we could get an ac vent in there!</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>data\images\hack_4147910648676056\img_1.jpg</t>
-        </is>
-      </c>
+          <t>Looking for recommendation on the best route (east to west) through Dallas /Ft Worth.   Midweek, hitting Dallas around Noon.  Pulling 36ft 5th wheel</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>RVhackcamp</t>
-        </is>
-      </c>
-      <c r="J49" t="n">
-        <v>4147910648676056</v>
-      </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/730771479_10102373262656439_2111230534189182674_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1206x952&amp;ctp=s640x640&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=DGSaV9gAmTAQ7kNvwEywMS_&amp;_nc_oc=AdprvPdL0g_5W2xgZVeuTA___ucidu0kEo0UPwtfNjLrGr8lzJOIt34RmN_8IoOdX94&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=05iOM0uUuQJ8MOIbywV40A&amp;_nc_ss=7b2a8&amp;oh=00_AQJbpgw45n6W01WKIaXHwonMf_0WGJsRiKeyxgsMLPAUaA&amp;oe=6AB3C7D6</t>
-        </is>
-      </c>
-      <c r="M49" t="n">
-        <v>1</v>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>أجهزة وإلكترونيات (Gadgets &amp; Power)</t>
-        </is>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>roadtreking</t>
+        </is>
+      </c>
+      <c r="K49" t="n">
+        <v>3359003754258580</v>
+      </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="n">
+        <v>0</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>rv 12v portable bunk fan</t>
-        </is>
-      </c>
-      <c r="P49" t="n">
-        <v>81</v>
-      </c>
-      <c r="Q49" t="inlineStr"/>
+          <t>غير مؤهل (بدون صور)</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="n">
+        <v>0</v>
+      </c>
+      <c r="R49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3466,43 +3625,50 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
+          <t>The bottom RV bunk used to be an absolute sauna until I found this on Amazon.
+Regular mini fans kept falling off, but this 12V fan clips on tight and actually pushes real air into that stuffy corner. My kids finally slept through the night!
+I'll drop the link in the first comment 👇</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
           <t>data\images\amazon_find_4147910648676056\img_1.jpg</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr">
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>4147910648676056</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr">
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/730771479_10102373262656439_2111230534189182674_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1206x952&amp;ctp=s640x640&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=DGSaV9gAmTAQ7kNvwEywMS_&amp;_nc_oc=AdprvPdL0g_5W2xgZVeuTA___ucidu0kEo0UPwtfNjLrGr8lzJOIt34RmN_8IoOdX94&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=-DNXGqSwxAYHz3InfHrB2g&amp;_nc_ss=7b2a8&amp;oh=00_AQKuI7NhSiWUW3pweIYcuSccGm2fBiXhQmnukqpjQKDiRg&amp;oe=6AB3C7D6</t>
         </is>
       </c>
-      <c r="M50" t="n">
+      <c r="N50" t="n">
         <v>1</v>
       </c>
-      <c r="N50" t="inlineStr">
+      <c r="O50" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr">
+      <c r="P50" t="inlineStr">
         <is>
           <t>rv 12v portable bunk fan</t>
         </is>
       </c>
-      <c r="P50" t="n">
+      <c r="Q50" t="n">
         <v>81</v>
       </c>
-      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3531,31 +3697,32 @@
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr">
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="K51" t="inlineStr">
         <is>
           <t>3359003754258580</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
-      <c r="M51" t="n">
-        <v>0</v>
-      </c>
-      <c r="N51" t="inlineStr">
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="n">
+        <v>0</v>
+      </c>
+      <c r="O51" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="n">
+        <v>0</v>
+      </c>
+      <c r="R51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3586,29 +3753,30 @@
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr">
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J52" t="n">
+      <c r="K52" t="n">
         <v>3629156827243270</v>
       </c>
-      <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
-      <c r="M52" t="n">
-        <v>0</v>
-      </c>
-      <c r="N52" t="inlineStr">
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="n">
+        <v>0</v>
+      </c>
+      <c r="O52" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="n">
+        <v>0</v>
+      </c>
+      <c r="R52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3639,31 +3807,32 @@
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr">
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="K53" t="inlineStr">
         <is>
           <t>3629156827243270</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr"/>
-      <c r="M53" t="n">
-        <v>0</v>
-      </c>
-      <c r="N53" t="inlineStr">
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O53" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="n">
+        <v>0</v>
+      </c>
+      <c r="R53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3692,29 +3861,30 @@
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr">
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J54" t="n">
+      <c r="K54" t="n">
         <v>3128604820606649</v>
       </c>
-      <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
-      <c r="M54" t="n">
-        <v>0</v>
-      </c>
-      <c r="N54" t="inlineStr">
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="n">
+        <v>0</v>
+      </c>
+      <c r="R54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3743,29 +3913,30 @@
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr">
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J55" t="n">
+      <c r="K55" t="n">
         <v>3617867058372247</v>
       </c>
-      <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
-      <c r="M55" t="n">
-        <v>0</v>
-      </c>
-      <c r="N55" t="inlineStr">
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="n">
+        <v>0</v>
+      </c>
+      <c r="R55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3794,31 +3965,32 @@
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr">
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="K56" t="inlineStr">
         <is>
           <t>3617867058372247</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr"/>
-      <c r="M56" t="n">
-        <v>0</v>
-      </c>
-      <c r="N56" t="inlineStr">
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q56" t="inlineStr"/>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="n">
+        <v>0</v>
+      </c>
+      <c r="R56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3847,31 +4019,32 @@
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr">
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
+      <c r="K57" t="inlineStr">
         <is>
           <t>3128604820606649</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr"/>
-      <c r="M57" t="n">
-        <v>0</v>
-      </c>
-      <c r="N57" t="inlineStr">
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q57" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="n">
+        <v>0</v>
+      </c>
+      <c r="R57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3900,31 +4073,32 @@
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr">
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
+      <c r="K58" t="inlineStr">
         <is>
           <t>3631536470338639</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
-      <c r="M58" t="n">
-        <v>0</v>
-      </c>
-      <c r="N58" t="inlineStr">
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="n">
+        <v>0</v>
+      </c>
+      <c r="R58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3953,29 +4127,30 @@
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr">
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J59" t="n">
+      <c r="K59" t="n">
         <v>3631536470338639</v>
       </c>
-      <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr"/>
-      <c r="M59" t="n">
-        <v>0</v>
-      </c>
-      <c r="N59" t="inlineStr">
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="n">
+        <v>0</v>
+      </c>
+      <c r="O59" t="inlineStr">
         <is>
           <t>غير مؤهل (بدون صور)</t>
         </is>
       </c>
-      <c r="O59" t="inlineStr"/>
-      <c r="P59" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q59" t="inlineStr"/>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="n">
+        <v>0</v>
+      </c>
+      <c r="R59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4003,39 +4178,40 @@
 Update: You all brought up a good question about draining the pool if it’s covering the shower drain. I’ve got a piece of 1” pvc pipe that’s about 18” long that I’m going to lay under it. Facing from the pool drain to the shower drain under the pool. I’m camping this week, so I’ll see how it goes.</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
         <is>
           <t>data\images\hack_2790989414393353\img_1.jpg; data\images\hack_2790989414393353\img_2.jpg</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr">
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J60" t="n">
+      <c r="K60" t="n">
         <v>2790989414393353</v>
       </c>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr">
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/516090961_10161909893284624_6283109645827272953_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx720x960&amp;ctp=s590x590&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=21QqBNNBMMcQ7kNvwFXmmny&amp;_nc_oc=AdrIEx__5typW7hR-DVpS1cS1KiVvk1PrfvUy26A3MGBEJcLOT0Oz5h4wAD_aTiMtdc&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=TuN4VeIUhMEDbkGyUlP9RA&amp;_nc_ss=7b2a8&amp;oh=00_AQLgKymahQgQWWDKDwUd5LluEkBVgZe5TCVyySuErcYTww&amp;oe=6AB39D03; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/516439294_10161909893409624_2902390173952908189_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx720x960&amp;ctp=s590x590&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=9TTZG7uN0nkQ7kNvwFOhIIY&amp;_nc_oc=AdqP8y920xXQBZnI0FoR2RcYpOQMVJtpls36tvoc7d_cT6Xch6Ir9FtebeM4WsSVGNo&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=TuN4VeIUhMEDbkGyUlP9RA&amp;_nc_ss=7b2a8&amp;oh=00_AQIV_O5dGMlir-2F0tzLrKDH1Pb9-zFmXcRrhC7qYi-1pA&amp;oe=6AB392A5</t>
         </is>
       </c>
-      <c r="M60" t="n">
-        <v>0</v>
-      </c>
-      <c r="N60" t="inlineStr">
+      <c r="N60" t="n">
+        <v>0</v>
+      </c>
+      <c r="O60" t="inlineStr">
         <is>
           <t>استبعاد (نقاش/سفر/شكوى)</t>
         </is>
       </c>
-      <c r="O60" t="inlineStr"/>
-      <c r="P60" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q60" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="n">
+        <v>0</v>
+      </c>
+      <c r="R60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4063,41 +4239,42 @@
 Update: You all brought up a good question about draining the pool if it’s covering the shower drain. I’ve got a piece of 1” pvc pipe that’s about 18” long that I’m going to lay under it. Facing from the pool drain to the shower drain under the pool. I’m camping this week, so I’ll see how it goes.</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr">
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr">
         <is>
           <t>data\images\hack_2790989414393353\img_1.jpg; data\images\hack_2790989414393353\img_2.jpg</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr">
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr">
+      <c r="K61" t="inlineStr">
         <is>
           <t>2790989414393353</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr">
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/516090961_10161909893284624_6283109645827272953_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx720x960&amp;ctp=s590x590&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=21QqBNNBMMcQ7kNvwFXmmny&amp;_nc_oc=AdrIEx__5typW7hR-DVpS1cS1KiVvk1PrfvUy26A3MGBEJcLOT0Oz5h4wAD_aTiMtdc&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=TuN4VeIUhMEDbkGyUlP9RA&amp;_nc_ss=7b2a8&amp;oh=00_AQLgKymahQgQWWDKDwUd5LluEkBVgZe5TCVyySuErcYTww&amp;oe=6AB39D03; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/516439294_10161909893409624_2902390173952908189_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx720x960&amp;ctp=s590x590&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=9TTZG7uN0nkQ7kNvwFOhIIY&amp;_nc_oc=AdqP8y920xXQBZnI0FoR2RcYpOQMVJtpls36tvoc7d_cT6Xch6Ir9FtebeM4WsSVGNo&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=TuN4VeIUhMEDbkGyUlP9RA&amp;_nc_ss=7b2a8&amp;oh=00_AQIV_O5dGMlir-2F0tzLrKDH1Pb9-zFmXcRrhC7qYi-1pA&amp;oe=6AB392A5</t>
         </is>
       </c>
-      <c r="M61" t="n">
-        <v>0</v>
-      </c>
-      <c r="N61" t="inlineStr">
+      <c r="N61" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" t="inlineStr">
         <is>
           <t>استبعاد (نقاش/سفر/شكوى)</t>
         </is>
       </c>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="n">
+        <v>0</v>
+      </c>
+      <c r="R61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4124,41 +4301,42 @@
           <t>Ok, maybe others have already done this but this was an inspiration my husband had for our new Class C. There is a stairwell that we worried we (or the dogs) would accidentally fall into. My hubby came up with this idea, I came up with the suggestion to staple one of Costco's rugs on it. To finish it off, so it could be easily moved aside, he attached handles and then screwed 2"x1" wood on the underside so it wouldn't move. I told him that he is brilliant! About a $33 project... عرض المزيد</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
         <is>
           <t>data\images\hack_3498835016916959\img_1.jpg; data\images\hack_3498835016916959\img_2.jpg; data\images\hack_3498835016916959\img_3.jpg</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr">
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="K62" t="inlineStr">
         <is>
           <t>3498835016916959</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr">
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/654206606_10233790263479320_8934352753678604081_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1186x843&amp;ctp=p417x417&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=6LvqWaRXDpoQ7kNvwHwFbcw&amp;_nc_oc=AdpRHF1lFIaB6-KwLOaxGwdKgH_HBUhvMtjzs-KH2Fc75eNwZYiKzaBQflOJ5FeGvI0&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQIsssXBVDsOtyPFbNnElRdrLu2szoLm7n1qTPnGMyvooQ&amp;oe=6AB3B55E; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/655884715_10233790268919456_2843537399331144636_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx881x828&amp;ctp=s590x590&amp;_nc_cat=104&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=tPEB8O9Kw8UQ7kNvwFZuVrV&amp;_nc_oc=AdqAr-YgIDyEtHOAEil6jSOgzA2VEFa-92RlVgLgi7BKPLYtkCurMvVl2nGViUNM7M4&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQIBieMdP15PfKQduK69kUkbIFthgt7oxQbZQJL2jWTmtw&amp;oe=6AB3A6A8; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/653720541_10233790263119311_2765445185799412382_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1204x904&amp;ctp=s590x590&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=oM21kLkiyXsQ7kNvwHrlGX5&amp;_nc_oc=AdosGU9wVGu-J4ks1YaFDknSu9pyGkNeKJ24PaDuDenJJ36LrD7FMNKTAobtawAnt7s&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQIERMSv9kKcWTY3PqqYJGPNgZ1dVK1fXzhW1DkB8pjJmg&amp;oe=6AB3C373</t>
         </is>
       </c>
-      <c r="M62" t="n">
-        <v>0</v>
-      </c>
-      <c r="N62" t="inlineStr">
+      <c r="N62" t="n">
+        <v>0</v>
+      </c>
+      <c r="O62" t="inlineStr">
         <is>
           <t>استبعاد (نقاش/سفر/شكوى)</t>
         </is>
       </c>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="n">
+        <v>0</v>
+      </c>
+      <c r="R62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4185,31 +4363,32 @@
           <t>Ok, maybe others have already done this but this was an inspiration my husband had for our new Class C. There is a stairwell that we worried we (or the dogs) would accidentally fall into. My hubby came up with this idea, I came up with the suggestion to staple one of Costco's rugs on it. To finish it off, so it could be easily moved aside, he attached handles and then screwed 2"x1" wood on the underside so it wouldn't move. I told him that he is brilliant! About a $33 project... عرض المزيد</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr">
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr">
         <is>
           <t>data\images\hack_3498835016916959\img_1.jpg; data\images\hack_3498835016916959\img_2.jpg; data\images\hack_3498835016916959\img_3.jpg</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr">
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr">
         <is>
           <t>RVhackcamp</t>
         </is>
       </c>
-      <c r="J63" t="n">
+      <c r="K63" t="n">
         <v>3498835016916959</v>
       </c>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr">
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/654206606_10233790263479320_8934352753678604081_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1186x843&amp;ctp=p417x417&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=6LvqWaRXDpoQ7kNvwHwFbcw&amp;_nc_oc=AdpRHF1lFIaB6-KwLOaxGwdKgH_HBUhvMtjzs-KH2Fc75eNwZYiKzaBQflOJ5FeGvI0&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQIsssXBVDsOtyPFbNnElRdrLu2szoLm7n1qTPnGMyvooQ&amp;oe=6AB3B55E; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/655884715_10233790268919456_2843537399331144636_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx881x828&amp;ctp=s590x590&amp;_nc_cat=104&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=tPEB8O9Kw8UQ7kNvwFZuVrV&amp;_nc_oc=AdqAr-YgIDyEtHOAEil6jSOgzA2VEFa-92RlVgLgi7BKPLYtkCurMvVl2nGViUNM7M4&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQIBieMdP15PfKQduK69kUkbIFthgt7oxQbZQJL2jWTmtw&amp;oe=6AB3A6A8; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/653720541_10233790263119311_2765445185799412382_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1204x904&amp;ctp=s590x590&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=oM21kLkiyXsQ7kNvwHrlGX5&amp;_nc_oc=AdosGU9wVGu-J4ks1YaFDknSu9pyGkNeKJ24PaDuDenJJ36LrD7FMNKTAobtawAnt7s&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=exjfy8yYqfVcO20J6DAxdQ&amp;_nc_ss=7b2a8&amp;oh=00_AQIERMSv9kKcWTY3PqqYJGPNgZ1dVK1fXzhW1DkB8pjJmg&amp;oe=6AB3C373</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr"/>
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr"/>
       <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4238,41 +4417,47 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
+          <t>Honestly didn't expect tailgate jack clearance flip to work this well, but it literally solved the problem on our last trip! Best purchase I've made in a while.
+I left the direct link in the first comment for anyone who needs it 👇</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
           <t>data\images\hack_3080238785468413\img_1.jpg; data\images\hack_3080238785468413\img_2.jpg</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr">
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J64" t="n">
+      <c r="K64" t="n">
         <v>3080238785468413</v>
       </c>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr">
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/500430078_3841916402724353_3119412760577639463_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=s590x590&amp;_nc_cat=103&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=3xqMlISBjIAQ7kNvwENGyA2&amp;_nc_oc=AdphwVhDvgBsBIiUyBGAqFab8JKFEBl-ecLqi4_6rvPomUH0laWqxzUXvA0Hp3F6cnE&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=TuN4VeIUhMEDbkGyUlP9RA&amp;_nc_ss=7b2a8&amp;oh=00_AQJiTLsbWgMHnDbD8AoTrKPQhartpGy2zgjUopRGh1QFmg&amp;oe=6AB3AAA4; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/500048722_3841913929391267_3300619833621540495_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=s590x590&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=-2TDJzpVcRAQ7kNvwFQnEva&amp;_nc_oc=AdpuXbdoq6LmiDAsXAmE89aFLUFHh2e5Fc4jb6FbXJLqE7s22JgyrfFYcSRJWFlKx7w&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=TuN4VeIUhMEDbkGyUlP9RA&amp;_nc_ss=7b2a8&amp;oh=00_AQLiyUu5lHeDHBi0WUR9hqUc5La82DyJVCGYjRR9HpYQxg&amp;oe=6AB3AB49</t>
         </is>
       </c>
-      <c r="M64" t="n">
+      <c r="N64" t="n">
         <v>1</v>
       </c>
-      <c r="N64" t="inlineStr">
+      <c r="O64" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O64" t="inlineStr">
+      <c r="P64" t="inlineStr">
         <is>
           <t>tailgate jack clearance flip</t>
         </is>
       </c>
-      <c r="P64" t="n">
+      <c r="Q64" t="n">
         <v>70</v>
       </c>
-      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4301,43 +4486,49 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
+          <t>Honestly didn't expect tailgate jack clearance flip to work this well, but it literally solved the problem on our last trip! Best purchase I've made in a while.
+I left the direct link in the first comment for anyone who needs it 👇</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
           <t>data\images\hack_3080238785468413\img_1.jpg; data\images\hack_3080238785468413\img_2.jpg</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr">
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr">
         <is>
           <t>roadtreking</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr">
+      <c r="K65" t="inlineStr">
         <is>
           <t>3080238785468413</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr">
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr">
         <is>
           <t>https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/500430078_3841916402724353_3119412760577639463_n.jpg?stp=dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=s590x590&amp;_nc_cat=103&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=3xqMlISBjIAQ7kNvwENGyA2&amp;_nc_oc=AdphwVhDvgBsBIiUyBGAqFab8JKFEBl-ecLqi4_6rvPomUH0laWqxzUXvA0Hp3F6cnE&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=TuN4VeIUhMEDbkGyUlP9RA&amp;_nc_ss=7b2a8&amp;oh=00_AQJiTLsbWgMHnDbD8AoTrKPQhartpGy2zgjUopRGh1QFmg&amp;oe=6AB3AAA4; https://scontent.fcai19-4.fna.fbcdn.net/v/t39.30808-6/500048722_3841913929391267_3300619833621540495_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1536x2048&amp;ctp=s590x590&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=aa7b47&amp;_nc_ohc=-2TDJzpVcRAQ7kNvwFQnEva&amp;_nc_oc=AdpuXbdoq6LmiDAsXAmE89aFLUFHh2e5Fc4jb6FbXJLqE7s22JgyrfFYcSRJWFlKx7w&amp;_nc_zt=23&amp;_nc_ht=scontent.fcai19-4.fna&amp;_nc_gid=TuN4VeIUhMEDbkGyUlP9RA&amp;_nc_ss=7b2a8&amp;oh=00_AQLiyUu5lHeDHBi0WUR9hqUc5La82DyJVCGYjRR9HpYQxg&amp;oe=6AB3AB49</t>
         </is>
       </c>
-      <c r="M65" t="n">
+      <c r="N65" t="n">
         <v>1</v>
       </c>
-      <c r="N65" t="inlineStr">
+      <c r="O65" t="inlineStr">
         <is>
           <t>أجهزة وإلكترونيات استهلاكية (Gadgets &amp; Appliances)</t>
         </is>
       </c>
-      <c r="O65" t="inlineStr">
+      <c r="P65" t="inlineStr">
         <is>
           <t>tailgate jack clearance flip</t>
         </is>
       </c>
-      <c r="P65" t="n">
+      <c r="Q65" t="n">
         <v>70</v>
       </c>
-      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>